<commit_message>
feat: re-run with draw figure
</commit_message>
<xml_diff>
--- a/results/final_0624_summary/Yeast_BinaryVector_summary.xlsx
+++ b/results/final_0624_summary/Yeast_BinaryVector_summary.xlsx
@@ -726,113 +726,281 @@
           <t>0.6570±0.0130</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>0.6267±0.0167</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>0.5029±0.0331</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>0.4067±0.0205</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>0.6890±0.0063</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0.6590±0.0106</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>0.5707±0.0136</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>0.4401±0.0109</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr">
         <is>
           <t>0.6848±0.0102</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>0.7116±0.0102</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>0.7698±0.0098</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>0.8460±0.0086</t>
+        </is>
+      </c>
       <c r="N2" t="inlineStr">
         <is>
           <t>0.6637±0.0059</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>0.6595±0.0080</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>0.6268±0.0084</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>0.5534±0.0087</t>
+        </is>
+      </c>
       <c r="R2" t="inlineStr">
         <is>
           <t>0.8064±0.0049</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>0.7905±0.0055</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>0.7275±0.0101</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>0.5901±0.0089</t>
+        </is>
+      </c>
       <c r="V2" t="inlineStr">
         <is>
           <t>0.5633±0.0072</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr"/>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>0.5527±0.0102</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>0.5030±0.0113</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>0.4089±0.0113</t>
+        </is>
+      </c>
       <c r="Z2" t="inlineStr">
         <is>
           <t>0.4323±0.0100</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>0.4439±0.0134</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>0.4541±0.0069</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>0.4422±0.0062</t>
+        </is>
+      </c>
       <c r="AD2" t="inlineStr">
         <is>
           <t>0.5469±0.0218</t>
         </is>
       </c>
-      <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>0.4710±0.0126</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>0.3893±0.0082</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>0.3394±0.0056</t>
+        </is>
+      </c>
       <c r="AH2" t="inlineStr">
         <is>
           <t>0.4327±0.0066</t>
         </is>
       </c>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
-      <c r="AK2" t="inlineStr"/>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>0.4659±0.0117</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>0.5540±0.0177</t>
+        </is>
+      </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>0.6991±0.0134</t>
+        </is>
+      </c>
       <c r="AL2" t="inlineStr">
         <is>
           <t>1.0000±0.0000</t>
         </is>
       </c>
-      <c r="AM2" t="inlineStr"/>
-      <c r="AN2" t="inlineStr"/>
-      <c r="AO2" t="inlineStr"/>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>0.9997±0.0008</t>
+        </is>
+      </c>
+      <c r="AN2" t="inlineStr">
+        <is>
+          <t>0.9986±0.0028</t>
+        </is>
+      </c>
+      <c r="AO2" t="inlineStr">
+        <is>
+          <t>0.9934±0.0061</t>
+        </is>
+      </c>
       <c r="AP2" t="inlineStr">
         <is>
           <t>0.6785±0.0068</t>
         </is>
       </c>
-      <c r="AQ2" t="inlineStr"/>
-      <c r="AR2" t="inlineStr"/>
-      <c r="AS2" t="inlineStr"/>
+      <c r="AQ2" t="inlineStr">
+        <is>
+          <t>0.6698±0.0086</t>
+        </is>
+      </c>
+      <c r="AR2" t="inlineStr">
+        <is>
+          <t>0.6291±0.0089</t>
+        </is>
+      </c>
+      <c r="AS2" t="inlineStr">
+        <is>
+          <t>0.5532±0.0062</t>
+        </is>
+      </c>
       <c r="AT2" t="inlineStr">
         <is>
           <t>0.6822±0.0076</t>
         </is>
       </c>
-      <c r="AU2" t="inlineStr"/>
-      <c r="AV2" t="inlineStr"/>
-      <c r="AW2" t="inlineStr"/>
+      <c r="AU2" t="inlineStr">
+        <is>
+          <t>0.6404±0.0100</t>
+        </is>
+      </c>
+      <c r="AV2" t="inlineStr">
+        <is>
+          <t>0.5352±0.0134</t>
+        </is>
+      </c>
+      <c r="AW2" t="inlineStr">
+        <is>
+          <t>0.4128±0.0068</t>
+        </is>
+      </c>
       <c r="AX2" t="inlineStr">
         <is>
           <t>0.6751±0.0111</t>
         </is>
       </c>
-      <c r="AY2" t="inlineStr"/>
-      <c r="AZ2" t="inlineStr"/>
-      <c r="BA2" t="inlineStr"/>
+      <c r="AY2" t="inlineStr">
+        <is>
+          <t>0.7023±0.0139</t>
+        </is>
+      </c>
+      <c r="AZ2" t="inlineStr">
+        <is>
+          <t>0.7634±0.0124</t>
+        </is>
+      </c>
+      <c r="BA2" t="inlineStr">
+        <is>
+          <t>0.8385±0.0103</t>
+        </is>
+      </c>
       <c r="BB2" t="inlineStr">
         <is>
           <t>0.2309±0.0199</t>
         </is>
       </c>
-      <c r="BC2" t="inlineStr"/>
-      <c r="BD2" t="inlineStr"/>
-      <c r="BE2" t="inlineStr"/>
+      <c r="BC2" t="inlineStr">
+        <is>
+          <t>0.1909±0.0215</t>
+        </is>
+      </c>
+      <c r="BD2" t="inlineStr">
+        <is>
+          <t>0.1020±0.0171</t>
+        </is>
+      </c>
+      <c r="BE2" t="inlineStr">
+        <is>
+          <t>0.0226±0.0135</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -845,113 +1013,281 @@
           <t>0.6603±0.0109</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>0.6287±0.0166</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0.5046±0.0320</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0.4132±0.0206</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>0.6795±0.0084</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0.6508±0.0108</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>0.5655±0.0140</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>0.4369±0.0102</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr">
         <is>
           <t>0.7099±0.0108</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>0.7242±0.0106</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>0.7792±0.0079</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>0.8501±0.0082</t>
+        </is>
+      </c>
       <c r="N3" t="inlineStr">
         <is>
           <t>0.6715±0.0066</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>0.6613±0.0084</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>0.6274±0.0090</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>0.5525±0.0083</t>
+        </is>
+      </c>
       <c r="R3" t="inlineStr">
         <is>
           <t>0.8053±0.0058</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>0.7880±0.0059</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>0.7255±0.0107</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>0.5879±0.0092</t>
+        </is>
+      </c>
       <c r="V3" t="inlineStr">
         <is>
           <t>0.5702±0.0078</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
-      <c r="Y3" t="inlineStr"/>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>0.5534±0.0104</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>0.5024±0.0119</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>0.4071±0.0105</t>
+        </is>
+      </c>
       <c r="Z3" t="inlineStr">
         <is>
           <t>0.4426±0.0090</t>
         </is>
       </c>
-      <c r="AA3" t="inlineStr"/>
-      <c r="AB3" t="inlineStr"/>
-      <c r="AC3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>0.4485±0.0127</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>0.4572±0.0077</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>0.4426±0.0063</t>
+        </is>
+      </c>
       <c r="AD3" t="inlineStr">
         <is>
           <t>0.5437±0.0196</t>
         </is>
       </c>
-      <c r="AE3" t="inlineStr"/>
-      <c r="AF3" t="inlineStr"/>
-      <c r="AG3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>0.4690±0.0101</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>0.3890±0.0092</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>0.3389±0.0057</t>
+        </is>
+      </c>
       <c r="AH3" t="inlineStr">
         <is>
           <t>0.4538±0.0073</t>
         </is>
       </c>
-      <c r="AI3" t="inlineStr"/>
-      <c r="AJ3" t="inlineStr"/>
-      <c r="AK3" t="inlineStr"/>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>0.4784±0.0108</t>
+        </is>
+      </c>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>0.5641±0.0170</t>
+        </is>
+      </c>
+      <c r="AK3" t="inlineStr">
+        <is>
+          <t>0.7036±0.0147</t>
+        </is>
+      </c>
       <c r="AL3" t="inlineStr">
         <is>
           <t>1.0000±0.0000</t>
         </is>
       </c>
-      <c r="AM3" t="inlineStr"/>
-      <c r="AN3" t="inlineStr"/>
-      <c r="AO3" t="inlineStr"/>
+      <c r="AM3" t="inlineStr">
+        <is>
+          <t>1.0000±0.0000</t>
+        </is>
+      </c>
+      <c r="AN3" t="inlineStr">
+        <is>
+          <t>0.9989±0.0025</t>
+        </is>
+      </c>
+      <c r="AO3" t="inlineStr">
+        <is>
+          <t>0.9942±0.0060</t>
+        </is>
+      </c>
       <c r="AP3" t="inlineStr">
         <is>
           <t>0.6847±0.0078</t>
         </is>
       </c>
-      <c r="AQ3" t="inlineStr"/>
-      <c r="AR3" t="inlineStr"/>
-      <c r="AS3" t="inlineStr"/>
+      <c r="AQ3" t="inlineStr">
+        <is>
+          <t>0.6712±0.0086</t>
+        </is>
+      </c>
+      <c r="AR3" t="inlineStr">
+        <is>
+          <t>0.6303±0.0096</t>
+        </is>
+      </c>
+      <c r="AS3" t="inlineStr">
+        <is>
+          <t>0.5532±0.0062</t>
+        </is>
+      </c>
       <c r="AT3" t="inlineStr">
         <is>
           <t>0.6715±0.0097</t>
         </is>
       </c>
-      <c r="AU3" t="inlineStr"/>
-      <c r="AV3" t="inlineStr"/>
-      <c r="AW3" t="inlineStr"/>
+      <c r="AU3" t="inlineStr">
+        <is>
+          <t>0.6325±0.0096</t>
+        </is>
+      </c>
+      <c r="AV3" t="inlineStr">
+        <is>
+          <t>0.5324±0.0139</t>
+        </is>
+      </c>
+      <c r="AW3" t="inlineStr">
+        <is>
+          <t>0.4117±0.0068</t>
+        </is>
+      </c>
       <c r="AX3" t="inlineStr">
         <is>
           <t>0.6985±0.0118</t>
         </is>
       </c>
-      <c r="AY3" t="inlineStr"/>
-      <c r="AZ3" t="inlineStr"/>
-      <c r="BA3" t="inlineStr"/>
+      <c r="AY3" t="inlineStr">
+        <is>
+          <t>0.7152±0.0132</t>
+        </is>
+      </c>
+      <c r="AZ3" t="inlineStr">
+        <is>
+          <t>0.7729±0.0108</t>
+        </is>
+      </c>
+      <c r="BA3" t="inlineStr">
+        <is>
+          <t>0.8428±0.0102</t>
+        </is>
+      </c>
       <c r="BB3" t="inlineStr">
         <is>
           <t>0.2242±0.0208</t>
         </is>
       </c>
-      <c r="BC3" t="inlineStr"/>
-      <c r="BD3" t="inlineStr"/>
-      <c r="BE3" t="inlineStr"/>
+      <c r="BC3" t="inlineStr">
+        <is>
+          <t>0.1791±0.0181</t>
+        </is>
+      </c>
+      <c r="BD3" t="inlineStr">
+        <is>
+          <t>0.0923±0.0145</t>
+        </is>
+      </c>
+      <c r="BE3" t="inlineStr">
+        <is>
+          <t>0.0159±0.0096</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -964,113 +1300,281 @@
           <t>0.6562±0.0128</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>0.6266±0.0166</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>0.5022±0.0324</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>0.4068±0.0204</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
           <t>0.6880±0.0061</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>0.6588±0.0108</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>0.5708±0.0134</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>0.4400±0.0108</t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr">
         <is>
           <t>0.6849±0.0093</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>0.7115±0.0102</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>0.7699±0.0097</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>0.8461±0.0085</t>
+        </is>
+      </c>
       <c r="N4" t="inlineStr">
         <is>
           <t>0.6636±0.0057</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>0.6594±0.0081</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>0.6268±0.0084</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>0.5533±0.0086</t>
+        </is>
+      </c>
       <c r="R4" t="inlineStr">
         <is>
           <t>0.8062±0.0049</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>0.7904±0.0055</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>0.7275±0.0102</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>0.5900±0.0088</t>
+        </is>
+      </c>
       <c r="V4" t="inlineStr">
         <is>
           <t>0.5632±0.0073</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="inlineStr"/>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>0.5526±0.0102</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>0.5030±0.0112</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>0.4088±0.0113</t>
+        </is>
+      </c>
       <c r="Z4" t="inlineStr">
         <is>
           <t>0.4326±0.0099</t>
         </is>
       </c>
-      <c r="AA4" t="inlineStr"/>
-      <c r="AB4" t="inlineStr"/>
-      <c r="AC4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>0.4438±0.0134</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>0.4545±0.0063</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>0.4422±0.0061</t>
+        </is>
+      </c>
       <c r="AD4" t="inlineStr">
         <is>
           <t>0.5465±0.0219</t>
         </is>
       </c>
-      <c r="AE4" t="inlineStr"/>
-      <c r="AF4" t="inlineStr"/>
-      <c r="AG4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>0.4709±0.0129</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>0.3896±0.0082</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>0.3394±0.0055</t>
+        </is>
+      </c>
       <c r="AH4" t="inlineStr">
         <is>
           <t>0.4332±0.0062</t>
         </is>
       </c>
-      <c r="AI4" t="inlineStr"/>
-      <c r="AJ4" t="inlineStr"/>
-      <c r="AK4" t="inlineStr"/>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>0.4659±0.0115</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>0.5543±0.0175</t>
+        </is>
+      </c>
+      <c r="AK4" t="inlineStr">
+        <is>
+          <t>0.6992±0.0134</t>
+        </is>
+      </c>
       <c r="AL4" t="inlineStr">
         <is>
           <t>1.0000±0.0000</t>
         </is>
       </c>
-      <c r="AM4" t="inlineStr"/>
-      <c r="AN4" t="inlineStr"/>
-      <c r="AO4" t="inlineStr"/>
+      <c r="AM4" t="inlineStr">
+        <is>
+          <t>0.9997±0.0008</t>
+        </is>
+      </c>
+      <c r="AN4" t="inlineStr">
+        <is>
+          <t>0.9981±0.0028</t>
+        </is>
+      </c>
+      <c r="AO4" t="inlineStr">
+        <is>
+          <t>0.9934±0.0061</t>
+        </is>
+      </c>
       <c r="AP4" t="inlineStr">
         <is>
           <t>0.6784±0.0067</t>
         </is>
       </c>
-      <c r="AQ4" t="inlineStr"/>
-      <c r="AR4" t="inlineStr"/>
-      <c r="AS4" t="inlineStr"/>
+      <c r="AQ4" t="inlineStr">
+        <is>
+          <t>0.6696±0.0086</t>
+        </is>
+      </c>
+      <c r="AR4" t="inlineStr">
+        <is>
+          <t>0.6292±0.0089</t>
+        </is>
+      </c>
+      <c r="AS4" t="inlineStr">
+        <is>
+          <t>0.5531±0.0061</t>
+        </is>
+      </c>
       <c r="AT4" t="inlineStr">
         <is>
           <t>0.6815±0.0076</t>
         </is>
       </c>
-      <c r="AU4" t="inlineStr"/>
-      <c r="AV4" t="inlineStr"/>
-      <c r="AW4" t="inlineStr"/>
+      <c r="AU4" t="inlineStr">
+        <is>
+          <t>0.6402±0.0102</t>
+        </is>
+      </c>
+      <c r="AV4" t="inlineStr">
+        <is>
+          <t>0.5353±0.0134</t>
+        </is>
+      </c>
+      <c r="AW4" t="inlineStr">
+        <is>
+          <t>0.4127±0.0067</t>
+        </is>
+      </c>
       <c r="AX4" t="inlineStr">
         <is>
           <t>0.6755±0.0107</t>
         </is>
       </c>
-      <c r="AY4" t="inlineStr"/>
-      <c r="AZ4" t="inlineStr"/>
-      <c r="BA4" t="inlineStr"/>
+      <c r="AY4" t="inlineStr">
+        <is>
+          <t>0.7021±0.0137</t>
+        </is>
+      </c>
+      <c r="AZ4" t="inlineStr">
+        <is>
+          <t>0.7636±0.0126</t>
+        </is>
+      </c>
+      <c r="BA4" t="inlineStr">
+        <is>
+          <t>0.8385±0.0105</t>
+        </is>
+      </c>
       <c r="BB4" t="inlineStr">
         <is>
           <t>0.2313±0.0201</t>
         </is>
       </c>
-      <c r="BC4" t="inlineStr"/>
-      <c r="BD4" t="inlineStr"/>
-      <c r="BE4" t="inlineStr"/>
+      <c r="BC4" t="inlineStr">
+        <is>
+          <t>0.1916±0.0213</t>
+        </is>
+      </c>
+      <c r="BD4" t="inlineStr">
+        <is>
+          <t>0.1022±0.0168</t>
+        </is>
+      </c>
+      <c r="BE4" t="inlineStr">
+        <is>
+          <t>0.0226±0.0135</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1083,113 +1587,281 @@
           <t>0.6610±0.0104</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>0.6292±0.0164</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>0.5053±0.0316</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>0.4133±0.0205</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>0.6788±0.0081</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>0.6507±0.0108</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>0.5652±0.0140</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>0.4366±0.0102</t>
+        </is>
+      </c>
       <c r="J5" t="inlineStr">
         <is>
           <t>0.7093±0.0104</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>0.7241±0.0106</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>0.7789±0.0082</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>0.8501±0.0084</t>
+        </is>
+      </c>
       <c r="N5" t="inlineStr">
         <is>
           <t>0.6709±0.0062</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>0.6612±0.0084</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>0.6271±0.0090</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>0.5523±0.0083</t>
+        </is>
+      </c>
       <c r="R5" t="inlineStr">
         <is>
           <t>0.8048±0.0055</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>0.7879±0.0058</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>0.7253±0.0107</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>0.5877±0.0091</t>
+        </is>
+      </c>
       <c r="V5" t="inlineStr">
         <is>
           <t>0.5695±0.0072</t>
         </is>
       </c>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
-      <c r="Y5" t="inlineStr"/>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>0.5533±0.0104</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>0.5021±0.0118</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>0.4068±0.0105</t>
+        </is>
+      </c>
       <c r="Z5" t="inlineStr">
         <is>
           <t>0.4417±0.0089</t>
         </is>
       </c>
-      <c r="AA5" t="inlineStr"/>
-      <c r="AB5" t="inlineStr"/>
-      <c r="AC5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>0.4481±0.0126</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>0.4567±0.0073</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>0.4424±0.0063</t>
+        </is>
+      </c>
       <c r="AD5" t="inlineStr">
         <is>
           <t>0.5408±0.0179</t>
         </is>
       </c>
-      <c r="AE5" t="inlineStr"/>
-      <c r="AF5" t="inlineStr"/>
-      <c r="AG5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>0.4683±0.0097</t>
+        </is>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>0.3885±0.0088</t>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>0.3388±0.0056</t>
+        </is>
+      </c>
       <c r="AH5" t="inlineStr">
         <is>
           <t>0.4532±0.0068</t>
         </is>
       </c>
-      <c r="AI5" t="inlineStr"/>
-      <c r="AJ5" t="inlineStr"/>
-      <c r="AK5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr">
+        <is>
+          <t>0.4781±0.0109</t>
+        </is>
+      </c>
+      <c r="AJ5" t="inlineStr">
+        <is>
+          <t>0.5636±0.0171</t>
+        </is>
+      </c>
+      <c r="AK5" t="inlineStr">
+        <is>
+          <t>0.7035±0.0147</t>
+        </is>
+      </c>
       <c r="AL5" t="inlineStr">
         <is>
           <t>1.0000±0.0000</t>
         </is>
       </c>
-      <c r="AM5" t="inlineStr"/>
-      <c r="AN5" t="inlineStr"/>
-      <c r="AO5" t="inlineStr"/>
+      <c r="AM5" t="inlineStr">
+        <is>
+          <t>1.0000±0.0000</t>
+        </is>
+      </c>
+      <c r="AN5" t="inlineStr">
+        <is>
+          <t>0.9989±0.0025</t>
+        </is>
+      </c>
+      <c r="AO5" t="inlineStr">
+        <is>
+          <t>0.9942±0.0060</t>
+        </is>
+      </c>
       <c r="AP5" t="inlineStr">
         <is>
           <t>0.6840±0.0074</t>
         </is>
       </c>
-      <c r="AQ5" t="inlineStr"/>
-      <c r="AR5" t="inlineStr"/>
-      <c r="AS5" t="inlineStr"/>
+      <c r="AQ5" t="inlineStr">
+        <is>
+          <t>0.6711±0.0085</t>
+        </is>
+      </c>
+      <c r="AR5" t="inlineStr">
+        <is>
+          <t>0.6300±0.0095</t>
+        </is>
+      </c>
+      <c r="AS5" t="inlineStr">
+        <is>
+          <t>0.5530±0.0061</t>
+        </is>
+      </c>
       <c r="AT5" t="inlineStr">
         <is>
           <t>0.6707±0.0093</t>
         </is>
       </c>
-      <c r="AU5" t="inlineStr"/>
-      <c r="AV5" t="inlineStr"/>
-      <c r="AW5" t="inlineStr"/>
+      <c r="AU5" t="inlineStr">
+        <is>
+          <t>0.6324±0.0095</t>
+        </is>
+      </c>
+      <c r="AV5" t="inlineStr">
+        <is>
+          <t>0.5321±0.0138</t>
+        </is>
+      </c>
+      <c r="AW5" t="inlineStr">
+        <is>
+          <t>0.4116±0.0067</t>
+        </is>
+      </c>
       <c r="AX5" t="inlineStr">
         <is>
           <t>0.6979±0.0113</t>
         </is>
       </c>
-      <c r="AY5" t="inlineStr"/>
-      <c r="AZ5" t="inlineStr"/>
-      <c r="BA5" t="inlineStr"/>
+      <c r="AY5" t="inlineStr">
+        <is>
+          <t>0.7150±0.0131</t>
+        </is>
+      </c>
+      <c r="AZ5" t="inlineStr">
+        <is>
+          <t>0.7727±0.0110</t>
+        </is>
+      </c>
+      <c r="BA5" t="inlineStr">
+        <is>
+          <t>0.8428±0.0104</t>
+        </is>
+      </c>
       <c r="BB5" t="inlineStr">
         <is>
           <t>0.2242±0.0196</t>
         </is>
       </c>
-      <c r="BC5" t="inlineStr"/>
-      <c r="BD5" t="inlineStr"/>
-      <c r="BE5" t="inlineStr"/>
+      <c r="BC5" t="inlineStr">
+        <is>
+          <t>0.1791±0.0184</t>
+        </is>
+      </c>
+      <c r="BD5" t="inlineStr">
+        <is>
+          <t>0.0923±0.0146</t>
+        </is>
+      </c>
+      <c r="BE5" t="inlineStr">
+        <is>
+          <t>0.0155±0.0093</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1202,113 +1874,281 @@
           <t>0.7456±0.0120</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>0.7434±0.0117</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>0.7311±0.0159</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0.6613±0.0155</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
           <t>0.7328±0.0084</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>0.7276±0.0084</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>0.7103±0.0094</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>0.6613±0.0110</t>
+        </is>
+      </c>
       <c r="J6" t="inlineStr">
         <is>
           <t>0.6002±0.0129</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>0.6003±0.0119</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>0.6015±0.0162</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>0.6211±0.0102</t>
+        </is>
+      </c>
       <c r="N6" t="inlineStr">
         <is>
           <t>0.6319±0.0076</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>0.6304±0.0075</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>0.6246±0.0079</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>0.6158±0.0059</t>
+        </is>
+      </c>
       <c r="R6" t="inlineStr">
         <is>
           <t>0.8129±0.0040</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>0.8102±0.0041</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>0.8033±0.0047</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>0.7836±0.0058</t>
+        </is>
+      </c>
       <c r="V6" t="inlineStr">
         <is>
           <t>0.5295±0.0075</t>
         </is>
       </c>
-      <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr"/>
-      <c r="Y6" t="inlineStr"/>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>0.5258±0.0092</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>0.5169±0.0098</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>0.4996±0.0096</t>
+        </is>
+      </c>
       <c r="Z6" t="inlineStr">
         <is>
           <t>0.3791±0.0081</t>
         </is>
       </c>
-      <c r="AA6" t="inlineStr"/>
-      <c r="AB6" t="inlineStr"/>
-      <c r="AC6" t="inlineStr"/>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>0.3739±0.0089</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>0.3735±0.0107</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>0.3894±0.0063</t>
+        </is>
+      </c>
       <c r="AD6" t="inlineStr">
         <is>
           <t>0.6452±0.0624</t>
         </is>
       </c>
-      <c r="AE6" t="inlineStr"/>
-      <c r="AF6" t="inlineStr"/>
-      <c r="AG6" t="inlineStr"/>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>0.6215±0.0547</t>
+        </is>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>0.5549±0.0493</t>
+        </is>
+      </c>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>0.4592±0.0262</t>
+        </is>
+      </c>
       <c r="AH6" t="inlineStr">
         <is>
           <t>0.3516±0.0080</t>
         </is>
       </c>
-      <c r="AI6" t="inlineStr"/>
-      <c r="AJ6" t="inlineStr"/>
-      <c r="AK6" t="inlineStr"/>
+      <c r="AI6" t="inlineStr">
+        <is>
+          <t>0.3501±0.0084</t>
+        </is>
+      </c>
+      <c r="AJ6" t="inlineStr">
+        <is>
+          <t>0.3530±0.0125</t>
+        </is>
+      </c>
+      <c r="AK6" t="inlineStr">
+        <is>
+          <t>0.3828±0.0072</t>
+        </is>
+      </c>
       <c r="AL6" t="inlineStr">
         <is>
           <t>1.0000±0.0000</t>
         </is>
       </c>
-      <c r="AM6" t="inlineStr"/>
-      <c r="AN6" t="inlineStr"/>
-      <c r="AO6" t="inlineStr"/>
+      <c r="AM6" t="inlineStr">
+        <is>
+          <t>1.0000±0.0000</t>
+        </is>
+      </c>
+      <c r="AN6" t="inlineStr">
+        <is>
+          <t>0.9998±0.0006</t>
+        </is>
+      </c>
+      <c r="AO6" t="inlineStr">
+        <is>
+          <t>0.9929±0.0037</t>
+        </is>
+      </c>
       <c r="AP6" t="inlineStr">
         <is>
           <t>0.6573±0.0072</t>
         </is>
       </c>
-      <c r="AQ6" t="inlineStr"/>
-      <c r="AR6" t="inlineStr"/>
-      <c r="AS6" t="inlineStr"/>
+      <c r="AQ6" t="inlineStr">
+        <is>
+          <t>0.6538±0.0078</t>
+        </is>
+      </c>
+      <c r="AR6" t="inlineStr">
+        <is>
+          <t>0.6458±0.0087</t>
+        </is>
+      </c>
+      <c r="AS6" t="inlineStr">
+        <is>
+          <t>0.6318±0.0069</t>
+        </is>
+      </c>
       <c r="AT6" t="inlineStr">
         <is>
           <t>0.7376±0.0078</t>
         </is>
       </c>
-      <c r="AU6" t="inlineStr"/>
-      <c r="AV6" t="inlineStr"/>
-      <c r="AW6" t="inlineStr"/>
+      <c r="AU6" t="inlineStr">
+        <is>
+          <t>0.7296±0.0081</t>
+        </is>
+      </c>
+      <c r="AV6" t="inlineStr">
+        <is>
+          <t>0.7101±0.0102</t>
+        </is>
+      </c>
+      <c r="AW6" t="inlineStr">
+        <is>
+          <t>0.6516±0.0109</t>
+        </is>
+      </c>
       <c r="AX6" t="inlineStr">
         <is>
           <t>0.5930±0.0132</t>
         </is>
       </c>
-      <c r="AY6" t="inlineStr"/>
-      <c r="AZ6" t="inlineStr"/>
-      <c r="BA6" t="inlineStr"/>
+      <c r="AY6" t="inlineStr">
+        <is>
+          <t>0.5924±0.0131</t>
+        </is>
+      </c>
+      <c r="AZ6" t="inlineStr">
+        <is>
+          <t>0.5926±0.0173</t>
+        </is>
+      </c>
+      <c r="BA6" t="inlineStr">
+        <is>
+          <t>0.6135±0.0121</t>
+        </is>
+      </c>
       <c r="BB6" t="inlineStr">
         <is>
           <t>0.2003±0.0158</t>
         </is>
       </c>
-      <c r="BC6" t="inlineStr"/>
-      <c r="BD6" t="inlineStr"/>
-      <c r="BE6" t="inlineStr"/>
+      <c r="BC6" t="inlineStr">
+        <is>
+          <t>0.1891±0.0221</t>
+        </is>
+      </c>
+      <c r="BD6" t="inlineStr">
+        <is>
+          <t>0.1647±0.0277</t>
+        </is>
+      </c>
+      <c r="BE6" t="inlineStr">
+        <is>
+          <t>0.1227±0.0257</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1321,113 +2161,281 @@
           <t>0.6897±0.0141</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>0.6740±0.0177</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>0.6317±0.0205</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>0.5345±0.0390</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>0.6763±0.0083</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>0.6592±0.0121</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>0.6149±0.0133</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>0.5197±0.0124</t>
+        </is>
+      </c>
       <c r="J7" t="inlineStr">
         <is>
           <t>0.7002±0.0115</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>0.7149±0.0100</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>0.7430±0.0118</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>0.7849±0.0111</t>
+        </is>
+      </c>
       <c r="N7" t="inlineStr">
         <is>
           <t>0.6662±0.0051</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>0.6635±0.0082</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>0.6501±0.0089</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>0.6031±0.0088</t>
+        </is>
+      </c>
       <c r="R7" t="inlineStr">
         <is>
           <t>0.8042±0.0049</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>0.7964±0.0066</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>0.7733±0.0073</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>0.7043±0.0092</t>
+        </is>
+      </c>
       <c r="V7" t="inlineStr">
         <is>
           <t>0.5633±0.0057</t>
         </is>
       </c>
-      <c r="W7" t="inlineStr"/>
-      <c r="X7" t="inlineStr"/>
-      <c r="Y7" t="inlineStr"/>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>0.5557±0.0103</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>0.5326±0.0099</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>0.4653±0.0103</t>
+        </is>
+      </c>
       <c r="Z7" t="inlineStr">
         <is>
           <t>0.4256±0.0092</t>
         </is>
       </c>
-      <c r="AA7" t="inlineStr"/>
-      <c r="AB7" t="inlineStr"/>
-      <c r="AC7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>0.4296±0.0131</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>0.4389±0.0088</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>0.4403±0.0115</t>
+        </is>
+      </c>
       <c r="AD7" t="inlineStr">
         <is>
           <t>0.5841±0.0319</t>
         </is>
       </c>
-      <c r="AE7" t="inlineStr"/>
-      <c r="AF7" t="inlineStr"/>
-      <c r="AG7" t="inlineStr"/>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>0.5255±0.0245</t>
+        </is>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>0.4418±0.0168</t>
+        </is>
+      </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>0.3666±0.0104</t>
+        </is>
+      </c>
       <c r="AH7" t="inlineStr">
         <is>
           <t>0.4380±0.0091</t>
         </is>
       </c>
-      <c r="AI7" t="inlineStr"/>
-      <c r="AJ7" t="inlineStr"/>
-      <c r="AK7" t="inlineStr"/>
+      <c r="AI7" t="inlineStr">
+        <is>
+          <t>0.4544±0.0086</t>
+        </is>
+      </c>
+      <c r="AJ7" t="inlineStr">
+        <is>
+          <t>0.4912±0.0073</t>
+        </is>
+      </c>
+      <c r="AK7" t="inlineStr">
+        <is>
+          <t>0.5643±0.0172</t>
+        </is>
+      </c>
       <c r="AL7" t="inlineStr">
         <is>
           <t>1.0000±0.0000</t>
         </is>
       </c>
-      <c r="AM7" t="inlineStr"/>
-      <c r="AN7" t="inlineStr"/>
-      <c r="AO7" t="inlineStr"/>
+      <c r="AM7" t="inlineStr">
+        <is>
+          <t>1.0000±0.0000</t>
+        </is>
+      </c>
+      <c r="AN7" t="inlineStr">
+        <is>
+          <t>0.9997±0.0008</t>
+        </is>
+      </c>
+      <c r="AO7" t="inlineStr">
+        <is>
+          <t>0.9964±0.0047</t>
+        </is>
+      </c>
       <c r="AP7" t="inlineStr">
         <is>
           <t>0.6804±0.0060</t>
         </is>
       </c>
-      <c r="AQ7" t="inlineStr"/>
-      <c r="AR7" t="inlineStr"/>
-      <c r="AS7" t="inlineStr"/>
+      <c r="AQ7" t="inlineStr">
+        <is>
+          <t>0.6766±0.0085</t>
+        </is>
+      </c>
+      <c r="AR7" t="inlineStr">
+        <is>
+          <t>0.6617±0.0086</t>
+        </is>
+      </c>
+      <c r="AS7" t="inlineStr">
+        <is>
+          <t>0.6140±0.0083</t>
+        </is>
+      </c>
       <c r="AT7" t="inlineStr">
         <is>
           <t>0.6724±0.0091</t>
         </is>
       </c>
-      <c r="AU7" t="inlineStr"/>
-      <c r="AV7" t="inlineStr"/>
-      <c r="AW7" t="inlineStr"/>
+      <c r="AU7" t="inlineStr">
+        <is>
+          <t>0.6517±0.0118</t>
+        </is>
+      </c>
+      <c r="AV7" t="inlineStr">
+        <is>
+          <t>0.6036±0.0129</t>
+        </is>
+      </c>
+      <c r="AW7" t="inlineStr">
+        <is>
+          <t>0.5077±0.0106</t>
+        </is>
+      </c>
       <c r="AX7" t="inlineStr">
         <is>
           <t>0.6889±0.0115</t>
         </is>
       </c>
-      <c r="AY7" t="inlineStr"/>
-      <c r="AZ7" t="inlineStr"/>
-      <c r="BA7" t="inlineStr"/>
+      <c r="AY7" t="inlineStr">
+        <is>
+          <t>0.7036±0.0111</t>
+        </is>
+      </c>
+      <c r="AZ7" t="inlineStr">
+        <is>
+          <t>0.7324±0.0104</t>
+        </is>
+      </c>
+      <c r="BA7" t="inlineStr">
+        <is>
+          <t>0.7770±0.0121</t>
+        </is>
+      </c>
       <c r="BB7" t="inlineStr">
         <is>
           <t>0.2122±0.0188</t>
         </is>
       </c>
-      <c r="BC7" t="inlineStr"/>
-      <c r="BD7" t="inlineStr"/>
-      <c r="BE7" t="inlineStr"/>
+      <c r="BC7" t="inlineStr">
+        <is>
+          <t>0.1771±0.0226</t>
+        </is>
+      </c>
+      <c r="BD7" t="inlineStr">
+        <is>
+          <t>0.1084±0.0144</t>
+        </is>
+      </c>
+      <c r="BE7" t="inlineStr">
+        <is>
+          <t>0.0199±0.0095</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1440,113 +2448,281 @@
           <t>0.7758±0.0119</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>0.7706±0.0111</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>0.7542±0.0157</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>0.6752±0.0149</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
           <t>0.7404±0.0067</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0.7346±0.0063</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>0.7190±0.0098</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>0.6654±0.0109</t>
+        </is>
+      </c>
       <c r="J8" t="inlineStr">
         <is>
           <t>0.5714±0.0146</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>0.5733±0.0122</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>0.5788±0.0146</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>0.6007±0.0103</t>
+        </is>
+      </c>
       <c r="N8" t="inlineStr">
         <is>
           <t>0.6163±0.0091</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>0.6161±0.0081</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>0.6140±0.0072</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>0.6061±0.0066</t>
+        </is>
+      </c>
       <c r="R8" t="inlineStr">
         <is>
           <t>0.8101±0.0044</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr"/>
-      <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr"/>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>0.8079±0.0045</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>0.8023±0.0043</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>0.7821±0.0058</t>
+        </is>
+      </c>
       <c r="V8" t="inlineStr">
         <is>
           <t>0.5126±0.0095</t>
         </is>
       </c>
-      <c r="W8" t="inlineStr"/>
-      <c r="X8" t="inlineStr"/>
-      <c r="Y8" t="inlineStr"/>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>0.5097±0.0095</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>0.5049±0.0086</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>0.4891±0.0105</t>
+        </is>
+      </c>
       <c r="Z8" t="inlineStr">
         <is>
           <t>0.3604±0.0093</t>
         </is>
       </c>
-      <c r="AA8" t="inlineStr"/>
-      <c r="AB8" t="inlineStr"/>
-      <c r="AC8" t="inlineStr"/>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>0.3582±0.0102</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>0.3605±0.0094</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>0.3784±0.0068</t>
+        </is>
+      </c>
       <c r="AD8" t="inlineStr">
         <is>
           <t>0.6261±0.0679</t>
         </is>
       </c>
-      <c r="AE8" t="inlineStr"/>
-      <c r="AF8" t="inlineStr"/>
-      <c r="AG8" t="inlineStr"/>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>0.6292±0.0570</t>
+        </is>
+      </c>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>0.5549±0.0490</t>
+        </is>
+      </c>
+      <c r="AG8" t="inlineStr">
+        <is>
+          <t>0.4554±0.0235</t>
+        </is>
+      </c>
       <c r="AH8" t="inlineStr">
         <is>
           <t>0.3289±0.0085</t>
         </is>
       </c>
-      <c r="AI8" t="inlineStr"/>
-      <c r="AJ8" t="inlineStr"/>
-      <c r="AK8" t="inlineStr"/>
+      <c r="AI8" t="inlineStr">
+        <is>
+          <t>0.3290±0.0084</t>
+        </is>
+      </c>
+      <c r="AJ8" t="inlineStr">
+        <is>
+          <t>0.3346±0.0109</t>
+        </is>
+      </c>
+      <c r="AK8" t="inlineStr">
+        <is>
+          <t>0.3659±0.0077</t>
+        </is>
+      </c>
       <c r="AL8" t="inlineStr">
         <is>
           <t>1.0000±0.0000</t>
         </is>
       </c>
-      <c r="AM8" t="inlineStr"/>
-      <c r="AN8" t="inlineStr"/>
-      <c r="AO8" t="inlineStr"/>
+      <c r="AM8" t="inlineStr">
+        <is>
+          <t>1.0000±0.0000</t>
+        </is>
+      </c>
+      <c r="AN8" t="inlineStr">
+        <is>
+          <t>0.9998±0.0006</t>
+        </is>
+      </c>
+      <c r="AO8" t="inlineStr">
+        <is>
+          <t>0.9919±0.0033</t>
+        </is>
+      </c>
       <c r="AP8" t="inlineStr">
         <is>
           <t>0.6437±0.0084</t>
         </is>
       </c>
-      <c r="AQ8" t="inlineStr"/>
-      <c r="AR8" t="inlineStr"/>
-      <c r="AS8" t="inlineStr"/>
+      <c r="AQ8" t="inlineStr">
+        <is>
+          <t>0.6411±0.0083</t>
+        </is>
+      </c>
+      <c r="AR8" t="inlineStr">
+        <is>
+          <t>0.6358±0.0080</t>
+        </is>
+      </c>
+      <c r="AS8" t="inlineStr">
+        <is>
+          <t>0.6224±0.0074</t>
+        </is>
+      </c>
       <c r="AT8" t="inlineStr">
         <is>
           <t>0.7449±0.0060</t>
         </is>
       </c>
-      <c r="AU8" t="inlineStr"/>
-      <c r="AV8" t="inlineStr"/>
-      <c r="AW8" t="inlineStr"/>
+      <c r="AU8" t="inlineStr">
+        <is>
+          <t>0.7376±0.0061</t>
+        </is>
+      </c>
+      <c r="AV8" t="inlineStr">
+        <is>
+          <t>0.7186±0.0106</t>
+        </is>
+      </c>
+      <c r="AW8" t="inlineStr">
+        <is>
+          <t>0.6546±0.0110</t>
+        </is>
+      </c>
       <c r="AX8" t="inlineStr">
         <is>
           <t>0.5669±0.0142</t>
         </is>
       </c>
-      <c r="AY8" t="inlineStr"/>
-      <c r="AZ8" t="inlineStr"/>
-      <c r="BA8" t="inlineStr"/>
+      <c r="AY8" t="inlineStr">
+        <is>
+          <t>0.5670±0.0130</t>
+        </is>
+      </c>
+      <c r="AZ8" t="inlineStr">
+        <is>
+          <t>0.5706±0.0153</t>
+        </is>
+      </c>
+      <c r="BA8" t="inlineStr">
+        <is>
+          <t>0.5934±0.0122</t>
+        </is>
+      </c>
       <c r="BB8" t="inlineStr">
         <is>
           <t>0.1796±0.0146</t>
         </is>
       </c>
-      <c r="BC8" t="inlineStr"/>
-      <c r="BD8" t="inlineStr"/>
-      <c r="BE8" t="inlineStr"/>
+      <c r="BC8" t="inlineStr">
+        <is>
+          <t>0.1645±0.0197</t>
+        </is>
+      </c>
+      <c r="BD8" t="inlineStr">
+        <is>
+          <t>0.1485±0.0233</t>
+        </is>
+      </c>
+      <c r="BE8" t="inlineStr">
+        <is>
+          <t>0.1146±0.0276</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1559,113 +2735,281 @@
           <t>0.6898±0.0158</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>0.6744±0.0184</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>0.6309±0.0193</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>0.5322±0.0423</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
           <t>0.6773±0.0082</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>0.6592±0.0122</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>0.6152±0.0126</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>0.5192±0.0122</t>
+        </is>
+      </c>
       <c r="J9" t="inlineStr">
         <is>
           <t>0.6993±0.0121</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>0.7142±0.0101</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>0.7431±0.0113</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>0.7838±0.0114</t>
+        </is>
+      </c>
       <c r="N9" t="inlineStr">
         <is>
           <t>0.6664±0.0054</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>0.6631±0.0085</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>0.6504±0.0085</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>0.6025±0.0089</t>
+        </is>
+      </c>
       <c r="R9" t="inlineStr">
         <is>
           <t>0.8047±0.0050</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr"/>
-      <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr"/>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>0.7964±0.0069</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>0.7736±0.0072</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>0.7040±0.0089</t>
+        </is>
+      </c>
       <c r="V9" t="inlineStr">
         <is>
           <t>0.5635±0.0059</t>
         </is>
       </c>
-      <c r="W9" t="inlineStr"/>
-      <c r="X9" t="inlineStr"/>
-      <c r="Y9" t="inlineStr"/>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>0.5553±0.0104</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>0.5331±0.0093</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>0.4647±0.0103</t>
+        </is>
+      </c>
       <c r="Z9" t="inlineStr">
         <is>
           <t>0.4267±0.0097</t>
         </is>
       </c>
-      <c r="AA9" t="inlineStr"/>
-      <c r="AB9" t="inlineStr"/>
-      <c r="AC9" t="inlineStr"/>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>0.4288±0.0128</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>0.4398±0.0072</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>0.4402±0.0121</t>
+        </is>
+      </c>
       <c r="AD9" t="inlineStr">
         <is>
           <t>0.5870±0.0326</t>
         </is>
       </c>
-      <c r="AE9" t="inlineStr"/>
-      <c r="AF9" t="inlineStr"/>
-      <c r="AG9" t="inlineStr"/>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>0.5282±0.0258</t>
+        </is>
+      </c>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>0.4455±0.0141</t>
+        </is>
+      </c>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>0.3663±0.0104</t>
+        </is>
+      </c>
       <c r="AH9" t="inlineStr">
         <is>
           <t>0.4379±0.0094</t>
         </is>
       </c>
-      <c r="AI9" t="inlineStr"/>
-      <c r="AJ9" t="inlineStr"/>
-      <c r="AK9" t="inlineStr"/>
+      <c r="AI9" t="inlineStr">
+        <is>
+          <t>0.4535±0.0083</t>
+        </is>
+      </c>
+      <c r="AJ9" t="inlineStr">
+        <is>
+          <t>0.4916±0.0074</t>
+        </is>
+      </c>
+      <c r="AK9" t="inlineStr">
+        <is>
+          <t>0.5643±0.0178</t>
+        </is>
+      </c>
       <c r="AL9" t="inlineStr">
         <is>
           <t>1.0000±0.0000</t>
         </is>
       </c>
-      <c r="AM9" t="inlineStr"/>
-      <c r="AN9" t="inlineStr"/>
-      <c r="AO9" t="inlineStr"/>
+      <c r="AM9" t="inlineStr">
+        <is>
+          <t>1.0000±0.0000</t>
+        </is>
+      </c>
+      <c r="AN9" t="inlineStr">
+        <is>
+          <t>0.9997±0.0008</t>
+        </is>
+      </c>
+      <c r="AO9" t="inlineStr">
+        <is>
+          <t>0.9964±0.0047</t>
+        </is>
+      </c>
       <c r="AP9" t="inlineStr">
         <is>
           <t>0.6808±0.0061</t>
         </is>
       </c>
-      <c r="AQ9" t="inlineStr"/>
-      <c r="AR9" t="inlineStr"/>
-      <c r="AS9" t="inlineStr"/>
+      <c r="AQ9" t="inlineStr">
+        <is>
+          <t>0.6763±0.0089</t>
+        </is>
+      </c>
+      <c r="AR9" t="inlineStr">
+        <is>
+          <t>0.6620±0.0082</t>
+        </is>
+      </c>
+      <c r="AS9" t="inlineStr">
+        <is>
+          <t>0.6136±0.0085</t>
+        </is>
+      </c>
       <c r="AT9" t="inlineStr">
         <is>
           <t>0.6738±0.0089</t>
         </is>
       </c>
-      <c r="AU9" t="inlineStr"/>
-      <c r="AV9" t="inlineStr"/>
-      <c r="AW9" t="inlineStr"/>
+      <c r="AU9" t="inlineStr">
+        <is>
+          <t>0.6518±0.0119</t>
+        </is>
+      </c>
+      <c r="AV9" t="inlineStr">
+        <is>
+          <t>0.6040±0.0121</t>
+        </is>
+      </c>
+      <c r="AW9" t="inlineStr">
+        <is>
+          <t>0.5074±0.0105</t>
+        </is>
+      </c>
       <c r="AX9" t="inlineStr">
         <is>
           <t>0.6882±0.0116</t>
         </is>
       </c>
-      <c r="AY9" t="inlineStr"/>
-      <c r="AZ9" t="inlineStr"/>
-      <c r="BA9" t="inlineStr"/>
+      <c r="AY9" t="inlineStr">
+        <is>
+          <t>0.7029±0.0111</t>
+        </is>
+      </c>
+      <c r="AZ9" t="inlineStr">
+        <is>
+          <t>0.7325±0.0105</t>
+        </is>
+      </c>
+      <c r="BA9" t="inlineStr">
+        <is>
+          <t>0.7762±0.0129</t>
+        </is>
+      </c>
       <c r="BB9" t="inlineStr">
         <is>
           <t>0.2127±0.0204</t>
         </is>
       </c>
-      <c r="BC9" t="inlineStr"/>
-      <c r="BD9" t="inlineStr"/>
-      <c r="BE9" t="inlineStr"/>
+      <c r="BC9" t="inlineStr">
+        <is>
+          <t>0.1761±0.0221</t>
+        </is>
+      </c>
+      <c r="BD9" t="inlineStr">
+        <is>
+          <t>0.1084±0.0131</t>
+        </is>
+      </c>
+      <c r="BE9" t="inlineStr">
+        <is>
+          <t>0.0186±0.0096</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1678,113 +3022,281 @@
           <t>0.7799±0.0118</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>0.7738±0.0153</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>0.7496±0.0202</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>0.6818±0.0135</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
           <t>0.7393±0.0078</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>0.7313±0.0096</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>0.7112±0.0085</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>0.6628±0.0115</t>
+        </is>
+      </c>
       <c r="J10" t="inlineStr">
         <is>
           <t>0.5636±0.0121</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>0.5589±0.0140</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>0.5504±0.0122</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>0.5310±0.0141</t>
+        </is>
+      </c>
       <c r="N10" t="inlineStr">
         <is>
           <t>0.6093±0.0074</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>0.6047±0.0086</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>0.5913±0.0060</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>0.5577±0.0092</t>
+        </is>
+      </c>
       <c r="R10" t="inlineStr">
         <is>
           <t>0.8091±0.0040</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr"/>
-      <c r="T10" t="inlineStr"/>
-      <c r="U10" t="inlineStr"/>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>0.8059±0.0048</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>0.7975±0.0030</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>0.7746±0.0032</t>
+        </is>
+      </c>
       <c r="V10" t="inlineStr">
         <is>
           <t>0.5035±0.0095</t>
         </is>
       </c>
-      <c r="W10" t="inlineStr"/>
-      <c r="X10" t="inlineStr"/>
-      <c r="Y10" t="inlineStr"/>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>0.4966±0.0094</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>0.4803±0.0055</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>0.4393±0.0090</t>
+        </is>
+      </c>
       <c r="Z10" t="inlineStr">
         <is>
           <t>0.3626±0.0080</t>
         </is>
       </c>
-      <c r="AA10" t="inlineStr"/>
-      <c r="AB10" t="inlineStr"/>
-      <c r="AC10" t="inlineStr"/>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>0.3573±0.0107</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>0.3561±0.0104</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>0.3602±0.0105</t>
+        </is>
+      </c>
       <c r="AD10" t="inlineStr">
         <is>
           <t>0.6401±0.0548</t>
         </is>
       </c>
-      <c r="AE10" t="inlineStr"/>
-      <c r="AF10" t="inlineStr"/>
-      <c r="AG10" t="inlineStr"/>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>0.6218±0.0528</t>
+        </is>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>0.5597±0.0264</t>
+        </is>
+      </c>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>0.4618±0.0220</t>
+        </is>
+      </c>
       <c r="AH10" t="inlineStr">
         <is>
           <t>0.3247±0.0081</t>
         </is>
       </c>
-      <c r="AI10" t="inlineStr"/>
-      <c r="AJ10" t="inlineStr"/>
-      <c r="AK10" t="inlineStr"/>
+      <c r="AI10" t="inlineStr">
+        <is>
+          <t>0.3222±0.0105</t>
+        </is>
+      </c>
+      <c r="AJ10" t="inlineStr">
+        <is>
+          <t>0.3217±0.0115</t>
+        </is>
+      </c>
+      <c r="AK10" t="inlineStr">
+        <is>
+          <t>0.3265±0.0095</t>
+        </is>
+      </c>
       <c r="AL10" t="inlineStr">
         <is>
           <t>1.0000±0.0000</t>
         </is>
       </c>
-      <c r="AM10" t="inlineStr"/>
-      <c r="AN10" t="inlineStr"/>
-      <c r="AO10" t="inlineStr"/>
+      <c r="AM10" t="inlineStr">
+        <is>
+          <t>1.0000±0.0000</t>
+        </is>
+      </c>
+      <c r="AN10" t="inlineStr">
+        <is>
+          <t>0.9998±0.0006</t>
+        </is>
+      </c>
+      <c r="AO10" t="inlineStr">
+        <is>
+          <t>0.9945±0.0035</t>
+        </is>
+      </c>
       <c r="AP10" t="inlineStr">
         <is>
           <t>0.6392±0.0077</t>
         </is>
       </c>
-      <c r="AQ10" t="inlineStr"/>
-      <c r="AR10" t="inlineStr"/>
-      <c r="AS10" t="inlineStr"/>
+      <c r="AQ10" t="inlineStr">
+        <is>
+          <t>0.6340±0.0085</t>
+        </is>
+      </c>
+      <c r="AR10" t="inlineStr">
+        <is>
+          <t>0.6203±0.0051</t>
+        </is>
+      </c>
+      <c r="AS10" t="inlineStr">
+        <is>
+          <t>0.5859±0.0077</t>
+        </is>
+      </c>
       <c r="AT10" t="inlineStr">
         <is>
           <t>0.7469±0.0085</t>
         </is>
       </c>
-      <c r="AU10" t="inlineStr"/>
-      <c r="AV10" t="inlineStr"/>
-      <c r="AW10" t="inlineStr"/>
+      <c r="AU10" t="inlineStr">
+        <is>
+          <t>0.7385±0.0107</t>
+        </is>
+      </c>
+      <c r="AV10" t="inlineStr">
+        <is>
+          <t>0.7172±0.0111</t>
+        </is>
+      </c>
+      <c r="AW10" t="inlineStr">
+        <is>
+          <t>0.6599±0.0132</t>
+        </is>
+      </c>
       <c r="AX10" t="inlineStr">
         <is>
           <t>0.5589±0.0129</t>
         </is>
       </c>
-      <c r="AY10" t="inlineStr"/>
-      <c r="AZ10" t="inlineStr"/>
-      <c r="BA10" t="inlineStr"/>
+      <c r="AY10" t="inlineStr">
+        <is>
+          <t>0.5557±0.0146</t>
+        </is>
+      </c>
+      <c r="AZ10" t="inlineStr">
+        <is>
+          <t>0.5468±0.0128</t>
+        </is>
+      </c>
+      <c r="BA10" t="inlineStr">
+        <is>
+          <t>0.5271±0.0126</t>
+        </is>
+      </c>
       <c r="BB10" t="inlineStr">
         <is>
           <t>0.1667±0.0175</t>
         </is>
       </c>
-      <c r="BC10" t="inlineStr"/>
-      <c r="BD10" t="inlineStr"/>
-      <c r="BE10" t="inlineStr"/>
+      <c r="BC10" t="inlineStr">
+        <is>
+          <t>0.1506±0.0133</t>
+        </is>
+      </c>
+      <c r="BD10" t="inlineStr">
+        <is>
+          <t>0.1254±0.0115</t>
+        </is>
+      </c>
+      <c r="BE10" t="inlineStr">
+        <is>
+          <t>0.0782±0.0120</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1797,113 +3309,281 @@
           <t>0.7515±0.0154</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>0.7705±0.0141</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>0.7577±0.0057</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>0.6870±0.0191</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr">
         <is>
           <t>0.7275±0.0083</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>0.7327±0.0091</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>0.7184±0.0109</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>0.6629±0.0149</t>
+        </is>
+      </c>
       <c r="J11" t="inlineStr">
         <is>
           <t>0.5814±0.0182</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>0.5649±0.0139</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>0.5542±0.0086</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>0.5404±0.0100</t>
+        </is>
+      </c>
       <c r="N11" t="inlineStr">
         <is>
           <t>0.6117±0.0098</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>0.6044±0.0090</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>0.5955±0.0073</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>0.5647±0.0097</t>
+        </is>
+      </c>
       <c r="R11" t="inlineStr">
         <is>
           <t>0.8082±0.0049</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr"/>
-      <c r="T11" t="inlineStr"/>
-      <c r="U11" t="inlineStr"/>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>0.8069±0.0042</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>0.8002±0.0046</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>0.7762±0.0059</t>
+        </is>
+      </c>
       <c r="V11" t="inlineStr">
         <is>
           <t>0.5134±0.0102</t>
         </is>
       </c>
-      <c r="W11" t="inlineStr"/>
-      <c r="X11" t="inlineStr"/>
-      <c r="Y11" t="inlineStr"/>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>0.5018±0.0089</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>0.4880±0.0090</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>0.4474±0.0109</t>
+        </is>
+      </c>
       <c r="Z11" t="inlineStr">
         <is>
           <t>0.3793±0.0125</t>
         </is>
       </c>
-      <c r="AA11" t="inlineStr"/>
-      <c r="AB11" t="inlineStr"/>
-      <c r="AC11" t="inlineStr"/>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>0.3627±0.0110</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>0.3518±0.0128</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>0.3558±0.0097</t>
+        </is>
+      </c>
       <c r="AD11" t="inlineStr">
         <is>
           <t>0.6016±0.0616</t>
         </is>
       </c>
-      <c r="AE11" t="inlineStr"/>
-      <c r="AF11" t="inlineStr"/>
-      <c r="AG11" t="inlineStr"/>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>0.5999±0.0579</t>
+        </is>
+      </c>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>0.5680±0.0423</t>
+        </is>
+      </c>
+      <c r="AG11" t="inlineStr">
+        <is>
+          <t>0.4446±0.0216</t>
+        </is>
+      </c>
       <c r="AH11" t="inlineStr">
         <is>
           <t>0.3460±0.0121</t>
         </is>
       </c>
-      <c r="AI11" t="inlineStr"/>
-      <c r="AJ11" t="inlineStr"/>
-      <c r="AK11" t="inlineStr"/>
+      <c r="AI11" t="inlineStr">
+        <is>
+          <t>0.3278±0.0090</t>
+        </is>
+      </c>
+      <c r="AJ11" t="inlineStr">
+        <is>
+          <t>0.3201±0.0085</t>
+        </is>
+      </c>
+      <c r="AK11" t="inlineStr">
+        <is>
+          <t>0.3283±0.0087</t>
+        </is>
+      </c>
       <c r="AL11" t="inlineStr">
         <is>
           <t>1.0000±0.0000</t>
         </is>
       </c>
-      <c r="AM11" t="inlineStr"/>
-      <c r="AN11" t="inlineStr"/>
-      <c r="AO11" t="inlineStr"/>
+      <c r="AM11" t="inlineStr">
+        <is>
+          <t>1.0000±0.0000</t>
+        </is>
+      </c>
+      <c r="AN11" t="inlineStr">
+        <is>
+          <t>0.9998±0.0006</t>
+        </is>
+      </c>
+      <c r="AO11" t="inlineStr">
+        <is>
+          <t>0.9951±0.0039</t>
+        </is>
+      </c>
       <c r="AP11" t="inlineStr">
         <is>
           <t>0.6451±0.0088</t>
         </is>
       </c>
-      <c r="AQ11" t="inlineStr"/>
-      <c r="AR11" t="inlineStr"/>
-      <c r="AS11" t="inlineStr"/>
+      <c r="AQ11" t="inlineStr">
+        <is>
+          <t>0.6368±0.0075</t>
+        </is>
+      </c>
+      <c r="AR11" t="inlineStr">
+        <is>
+          <t>0.6246±0.0079</t>
+        </is>
+      </c>
+      <c r="AS11" t="inlineStr">
+        <is>
+          <t>0.5924±0.0086</t>
+        </is>
+      </c>
       <c r="AT11" t="inlineStr">
         <is>
           <t>0.7330±0.0055</t>
         </is>
       </c>
-      <c r="AU11" t="inlineStr"/>
-      <c r="AV11" t="inlineStr"/>
-      <c r="AW11" t="inlineStr"/>
+      <c r="AU11" t="inlineStr">
+        <is>
+          <t>0.7393±0.0073</t>
+        </is>
+      </c>
+      <c r="AV11" t="inlineStr">
+        <is>
+          <t>0.7243±0.0138</t>
+        </is>
+      </c>
+      <c r="AW11" t="inlineStr">
+        <is>
+          <t>0.6603±0.0143</t>
+        </is>
+      </c>
       <c r="AX11" t="inlineStr">
         <is>
           <t>0.5764±0.0161</t>
         </is>
       </c>
-      <c r="AY11" t="inlineStr"/>
-      <c r="AZ11" t="inlineStr"/>
-      <c r="BA11" t="inlineStr"/>
+      <c r="AY11" t="inlineStr">
+        <is>
+          <t>0.5594±0.0121</t>
+        </is>
+      </c>
+      <c r="AZ11" t="inlineStr">
+        <is>
+          <t>0.5491±0.0093</t>
+        </is>
+      </c>
+      <c r="BA11" t="inlineStr">
+        <is>
+          <t>0.5374±0.0103</t>
+        </is>
+      </c>
       <c r="BB11" t="inlineStr">
         <is>
           <t>0.2201±0.0155</t>
         </is>
       </c>
-      <c r="BC11" t="inlineStr"/>
-      <c r="BD11" t="inlineStr"/>
-      <c r="BE11" t="inlineStr"/>
+      <c r="BC11" t="inlineStr">
+        <is>
+          <t>0.1849±0.0154</t>
+        </is>
+      </c>
+      <c r="BD11" t="inlineStr">
+        <is>
+          <t>0.1487±0.0164</t>
+        </is>
+      </c>
+      <c r="BE11" t="inlineStr">
+        <is>
+          <t>0.0799±0.0161</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1916,113 +3596,281 @@
           <t>0.8898±0.0128</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>0.8847±0.0124</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>0.8710±0.0182</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>0.8217±0.0168</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr">
         <is>
           <t>0.7570±0.0106</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>0.7539±0.0076</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>0.7489±0.0096</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>0.7234±0.0133</t>
+        </is>
+      </c>
       <c r="J12" t="inlineStr">
         <is>
           <t>0.4481±0.0171</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>0.4611±0.0154</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>0.4556±0.0156</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>0.4287±0.0159</t>
+        </is>
+      </c>
       <c r="N12" t="inlineStr">
         <is>
           <t>0.5368±0.0131</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>0.5456±0.0109</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>0.5383±0.0114</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>0.5066±0.0140</t>
+        </is>
+      </c>
       <c r="R12" t="inlineStr">
         <is>
           <t>0.7930±0.0056</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr"/>
-      <c r="T12" t="inlineStr"/>
-      <c r="U12" t="inlineStr"/>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>0.7952±0.0052</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>0.7933±0.0060</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>0.7835±0.0050</t>
+        </is>
+      </c>
       <c r="V12" t="inlineStr">
         <is>
           <t>0.4227±0.0121</t>
         </is>
       </c>
-      <c r="W12" t="inlineStr"/>
-      <c r="X12" t="inlineStr"/>
-      <c r="Y12" t="inlineStr"/>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>0.4333±0.0112</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>0.4264±0.0123</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>0.3953±0.0134</t>
+        </is>
+      </c>
       <c r="Z12" t="inlineStr">
         <is>
           <t>0.2637±0.0120</t>
         </is>
       </c>
-      <c r="AA12" t="inlineStr"/>
-      <c r="AB12" t="inlineStr"/>
-      <c r="AC12" t="inlineStr"/>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>0.2718±0.0115</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>0.2713±0.0138</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>0.2720±0.0101</t>
+        </is>
+      </c>
       <c r="AD12" t="inlineStr">
         <is>
           <t>0.5934±0.0745</t>
         </is>
       </c>
-      <c r="AE12" t="inlineStr"/>
-      <c r="AF12" t="inlineStr"/>
-      <c r="AG12" t="inlineStr"/>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>0.5903±0.0697</t>
+        </is>
+      </c>
+      <c r="AF12" t="inlineStr">
+        <is>
+          <t>0.5447±0.0523</t>
+        </is>
+      </c>
+      <c r="AG12" t="inlineStr">
+        <is>
+          <t>0.5556±0.0786</t>
+        </is>
+      </c>
       <c r="AH12" t="inlineStr">
         <is>
           <t>0.2306±0.0089</t>
         </is>
       </c>
-      <c r="AI12" t="inlineStr"/>
-      <c r="AJ12" t="inlineStr"/>
-      <c r="AK12" t="inlineStr"/>
+      <c r="AI12" t="inlineStr">
+        <is>
+          <t>0.2395±0.0090</t>
+        </is>
+      </c>
+      <c r="AJ12" t="inlineStr">
+        <is>
+          <t>0.2373±0.0106</t>
+        </is>
+      </c>
+      <c r="AK12" t="inlineStr">
+        <is>
+          <t>0.2292±0.0097</t>
+        </is>
+      </c>
       <c r="AL12" t="inlineStr">
         <is>
           <t>1.0000±0.0000</t>
         </is>
       </c>
-      <c r="AM12" t="inlineStr"/>
-      <c r="AN12" t="inlineStr"/>
-      <c r="AO12" t="inlineStr"/>
+      <c r="AM12" t="inlineStr">
+        <is>
+          <t>1.0000±0.0000</t>
+        </is>
+      </c>
+      <c r="AN12" t="inlineStr">
+        <is>
+          <t>1.0000±0.0000</t>
+        </is>
+      </c>
+      <c r="AO12" t="inlineStr">
+        <is>
+          <t>1.0000±0.0000</t>
+        </is>
+      </c>
       <c r="AP12" t="inlineStr">
         <is>
           <t>0.5689±0.0119</t>
         </is>
       </c>
-      <c r="AQ12" t="inlineStr"/>
-      <c r="AR12" t="inlineStr"/>
-      <c r="AS12" t="inlineStr"/>
+      <c r="AQ12" t="inlineStr">
+        <is>
+          <t>0.5782±0.0110</t>
+        </is>
+      </c>
+      <c r="AR12" t="inlineStr">
+        <is>
+          <t>0.5721±0.0130</t>
+        </is>
+      </c>
+      <c r="AS12" t="inlineStr">
+        <is>
+          <t>0.5444±0.0129</t>
+        </is>
+      </c>
       <c r="AT12" t="inlineStr">
         <is>
           <t>0.7696±0.0084</t>
         </is>
       </c>
-      <c r="AU12" t="inlineStr"/>
-      <c r="AV12" t="inlineStr"/>
-      <c r="AW12" t="inlineStr"/>
+      <c r="AU12" t="inlineStr">
+        <is>
+          <t>0.7673±0.0083</t>
+        </is>
+      </c>
+      <c r="AV12" t="inlineStr">
+        <is>
+          <t>0.7659±0.0107</t>
+        </is>
+      </c>
+      <c r="AW12" t="inlineStr">
+        <is>
+          <t>0.7501±0.0138</t>
+        </is>
+      </c>
       <c r="AX12" t="inlineStr">
         <is>
           <t>0.4514±0.0142</t>
         </is>
       </c>
-      <c r="AY12" t="inlineStr"/>
-      <c r="AZ12" t="inlineStr"/>
-      <c r="BA12" t="inlineStr"/>
+      <c r="AY12" t="inlineStr">
+        <is>
+          <t>0.4640±0.0136</t>
+        </is>
+      </c>
+      <c r="AZ12" t="inlineStr">
+        <is>
+          <t>0.4568±0.0153</t>
+        </is>
+      </c>
+      <c r="BA12" t="inlineStr">
+        <is>
+          <t>0.4276±0.0172</t>
+        </is>
+      </c>
       <c r="BB12" t="inlineStr">
         <is>
           <t>0.0819±0.0095</t>
         </is>
       </c>
-      <c r="BC12" t="inlineStr"/>
-      <c r="BD12" t="inlineStr"/>
-      <c r="BE12" t="inlineStr"/>
+      <c r="BC12" t="inlineStr">
+        <is>
+          <t>0.0952±0.0143</t>
+        </is>
+      </c>
+      <c r="BD12" t="inlineStr">
+        <is>
+          <t>0.0923±0.0107</t>
+        </is>
+      </c>
+      <c r="BE12" t="inlineStr">
+        <is>
+          <t>0.0753±0.0156</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">

</xml_diff>

<commit_message>
feat: re-run with draw figure (#2)
</commit_message>
<xml_diff>
--- a/results/final_0624_summary/Yeast_BinaryVector_summary.xlsx
+++ b/results/final_0624_summary/Yeast_BinaryVector_summary.xlsx
@@ -726,113 +726,281 @@
           <t>0.6570±0.0130</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>0.6267±0.0167</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>0.5029±0.0331</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>0.4067±0.0205</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>0.6890±0.0063</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0.6590±0.0106</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>0.5707±0.0136</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>0.4401±0.0109</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr">
         <is>
           <t>0.6848±0.0102</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>0.7116±0.0102</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>0.7698±0.0098</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>0.8460±0.0086</t>
+        </is>
+      </c>
       <c r="N2" t="inlineStr">
         <is>
           <t>0.6637±0.0059</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>0.6595±0.0080</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>0.6268±0.0084</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>0.5534±0.0087</t>
+        </is>
+      </c>
       <c r="R2" t="inlineStr">
         <is>
           <t>0.8064±0.0049</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>0.7905±0.0055</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>0.7275±0.0101</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>0.5901±0.0089</t>
+        </is>
+      </c>
       <c r="V2" t="inlineStr">
         <is>
           <t>0.5633±0.0072</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr"/>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>0.5527±0.0102</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>0.5030±0.0113</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>0.4089±0.0113</t>
+        </is>
+      </c>
       <c r="Z2" t="inlineStr">
         <is>
           <t>0.4323±0.0100</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>0.4439±0.0134</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>0.4541±0.0069</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>0.4422±0.0062</t>
+        </is>
+      </c>
       <c r="AD2" t="inlineStr">
         <is>
           <t>0.5469±0.0218</t>
         </is>
       </c>
-      <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>0.4710±0.0126</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>0.3893±0.0082</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>0.3394±0.0056</t>
+        </is>
+      </c>
       <c r="AH2" t="inlineStr">
         <is>
           <t>0.4327±0.0066</t>
         </is>
       </c>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
-      <c r="AK2" t="inlineStr"/>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>0.4659±0.0117</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>0.5540±0.0177</t>
+        </is>
+      </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>0.6991±0.0134</t>
+        </is>
+      </c>
       <c r="AL2" t="inlineStr">
         <is>
           <t>1.0000±0.0000</t>
         </is>
       </c>
-      <c r="AM2" t="inlineStr"/>
-      <c r="AN2" t="inlineStr"/>
-      <c r="AO2" t="inlineStr"/>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>0.9997±0.0008</t>
+        </is>
+      </c>
+      <c r="AN2" t="inlineStr">
+        <is>
+          <t>0.9986±0.0028</t>
+        </is>
+      </c>
+      <c r="AO2" t="inlineStr">
+        <is>
+          <t>0.9934±0.0061</t>
+        </is>
+      </c>
       <c r="AP2" t="inlineStr">
         <is>
           <t>0.6785±0.0068</t>
         </is>
       </c>
-      <c r="AQ2" t="inlineStr"/>
-      <c r="AR2" t="inlineStr"/>
-      <c r="AS2" t="inlineStr"/>
+      <c r="AQ2" t="inlineStr">
+        <is>
+          <t>0.6698±0.0086</t>
+        </is>
+      </c>
+      <c r="AR2" t="inlineStr">
+        <is>
+          <t>0.6291±0.0089</t>
+        </is>
+      </c>
+      <c r="AS2" t="inlineStr">
+        <is>
+          <t>0.5532±0.0062</t>
+        </is>
+      </c>
       <c r="AT2" t="inlineStr">
         <is>
           <t>0.6822±0.0076</t>
         </is>
       </c>
-      <c r="AU2" t="inlineStr"/>
-      <c r="AV2" t="inlineStr"/>
-      <c r="AW2" t="inlineStr"/>
+      <c r="AU2" t="inlineStr">
+        <is>
+          <t>0.6404±0.0100</t>
+        </is>
+      </c>
+      <c r="AV2" t="inlineStr">
+        <is>
+          <t>0.5352±0.0134</t>
+        </is>
+      </c>
+      <c r="AW2" t="inlineStr">
+        <is>
+          <t>0.4128±0.0068</t>
+        </is>
+      </c>
       <c r="AX2" t="inlineStr">
         <is>
           <t>0.6751±0.0111</t>
         </is>
       </c>
-      <c r="AY2" t="inlineStr"/>
-      <c r="AZ2" t="inlineStr"/>
-      <c r="BA2" t="inlineStr"/>
+      <c r="AY2" t="inlineStr">
+        <is>
+          <t>0.7023±0.0139</t>
+        </is>
+      </c>
+      <c r="AZ2" t="inlineStr">
+        <is>
+          <t>0.7634±0.0124</t>
+        </is>
+      </c>
+      <c r="BA2" t="inlineStr">
+        <is>
+          <t>0.8385±0.0103</t>
+        </is>
+      </c>
       <c r="BB2" t="inlineStr">
         <is>
           <t>0.2309±0.0199</t>
         </is>
       </c>
-      <c r="BC2" t="inlineStr"/>
-      <c r="BD2" t="inlineStr"/>
-      <c r="BE2" t="inlineStr"/>
+      <c r="BC2" t="inlineStr">
+        <is>
+          <t>0.1909±0.0215</t>
+        </is>
+      </c>
+      <c r="BD2" t="inlineStr">
+        <is>
+          <t>0.1020±0.0171</t>
+        </is>
+      </c>
+      <c r="BE2" t="inlineStr">
+        <is>
+          <t>0.0226±0.0135</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -845,113 +1013,281 @@
           <t>0.6603±0.0109</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>0.6287±0.0166</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0.5046±0.0320</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0.4132±0.0206</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>0.6795±0.0084</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0.6508±0.0108</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>0.5655±0.0140</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>0.4369±0.0102</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr">
         <is>
           <t>0.7099±0.0108</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>0.7242±0.0106</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>0.7792±0.0079</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>0.8501±0.0082</t>
+        </is>
+      </c>
       <c r="N3" t="inlineStr">
         <is>
           <t>0.6715±0.0066</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>0.6613±0.0084</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>0.6274±0.0090</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>0.5525±0.0083</t>
+        </is>
+      </c>
       <c r="R3" t="inlineStr">
         <is>
           <t>0.8053±0.0058</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>0.7880±0.0059</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>0.7255±0.0107</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>0.5879±0.0092</t>
+        </is>
+      </c>
       <c r="V3" t="inlineStr">
         <is>
           <t>0.5702±0.0078</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
-      <c r="Y3" t="inlineStr"/>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>0.5534±0.0104</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>0.5024±0.0119</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>0.4071±0.0105</t>
+        </is>
+      </c>
       <c r="Z3" t="inlineStr">
         <is>
           <t>0.4426±0.0090</t>
         </is>
       </c>
-      <c r="AA3" t="inlineStr"/>
-      <c r="AB3" t="inlineStr"/>
-      <c r="AC3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>0.4485±0.0127</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>0.4572±0.0077</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>0.4426±0.0063</t>
+        </is>
+      </c>
       <c r="AD3" t="inlineStr">
         <is>
           <t>0.5437±0.0196</t>
         </is>
       </c>
-      <c r="AE3" t="inlineStr"/>
-      <c r="AF3" t="inlineStr"/>
-      <c r="AG3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>0.4690±0.0101</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>0.3890±0.0092</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>0.3389±0.0057</t>
+        </is>
+      </c>
       <c r="AH3" t="inlineStr">
         <is>
           <t>0.4538±0.0073</t>
         </is>
       </c>
-      <c r="AI3" t="inlineStr"/>
-      <c r="AJ3" t="inlineStr"/>
-      <c r="AK3" t="inlineStr"/>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>0.4784±0.0108</t>
+        </is>
+      </c>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>0.5641±0.0170</t>
+        </is>
+      </c>
+      <c r="AK3" t="inlineStr">
+        <is>
+          <t>0.7036±0.0147</t>
+        </is>
+      </c>
       <c r="AL3" t="inlineStr">
         <is>
           <t>1.0000±0.0000</t>
         </is>
       </c>
-      <c r="AM3" t="inlineStr"/>
-      <c r="AN3" t="inlineStr"/>
-      <c r="AO3" t="inlineStr"/>
+      <c r="AM3" t="inlineStr">
+        <is>
+          <t>1.0000±0.0000</t>
+        </is>
+      </c>
+      <c r="AN3" t="inlineStr">
+        <is>
+          <t>0.9989±0.0025</t>
+        </is>
+      </c>
+      <c r="AO3" t="inlineStr">
+        <is>
+          <t>0.9942±0.0060</t>
+        </is>
+      </c>
       <c r="AP3" t="inlineStr">
         <is>
           <t>0.6847±0.0078</t>
         </is>
       </c>
-      <c r="AQ3" t="inlineStr"/>
-      <c r="AR3" t="inlineStr"/>
-      <c r="AS3" t="inlineStr"/>
+      <c r="AQ3" t="inlineStr">
+        <is>
+          <t>0.6712±0.0086</t>
+        </is>
+      </c>
+      <c r="AR3" t="inlineStr">
+        <is>
+          <t>0.6303±0.0096</t>
+        </is>
+      </c>
+      <c r="AS3" t="inlineStr">
+        <is>
+          <t>0.5532±0.0062</t>
+        </is>
+      </c>
       <c r="AT3" t="inlineStr">
         <is>
           <t>0.6715±0.0097</t>
         </is>
       </c>
-      <c r="AU3" t="inlineStr"/>
-      <c r="AV3" t="inlineStr"/>
-      <c r="AW3" t="inlineStr"/>
+      <c r="AU3" t="inlineStr">
+        <is>
+          <t>0.6325±0.0096</t>
+        </is>
+      </c>
+      <c r="AV3" t="inlineStr">
+        <is>
+          <t>0.5324±0.0139</t>
+        </is>
+      </c>
+      <c r="AW3" t="inlineStr">
+        <is>
+          <t>0.4117±0.0068</t>
+        </is>
+      </c>
       <c r="AX3" t="inlineStr">
         <is>
           <t>0.6985±0.0118</t>
         </is>
       </c>
-      <c r="AY3" t="inlineStr"/>
-      <c r="AZ3" t="inlineStr"/>
-      <c r="BA3" t="inlineStr"/>
+      <c r="AY3" t="inlineStr">
+        <is>
+          <t>0.7152±0.0132</t>
+        </is>
+      </c>
+      <c r="AZ3" t="inlineStr">
+        <is>
+          <t>0.7729±0.0108</t>
+        </is>
+      </c>
+      <c r="BA3" t="inlineStr">
+        <is>
+          <t>0.8428±0.0102</t>
+        </is>
+      </c>
       <c r="BB3" t="inlineStr">
         <is>
           <t>0.2242±0.0208</t>
         </is>
       </c>
-      <c r="BC3" t="inlineStr"/>
-      <c r="BD3" t="inlineStr"/>
-      <c r="BE3" t="inlineStr"/>
+      <c r="BC3" t="inlineStr">
+        <is>
+          <t>0.1791±0.0181</t>
+        </is>
+      </c>
+      <c r="BD3" t="inlineStr">
+        <is>
+          <t>0.0923±0.0145</t>
+        </is>
+      </c>
+      <c r="BE3" t="inlineStr">
+        <is>
+          <t>0.0159±0.0096</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -964,113 +1300,281 @@
           <t>0.6562±0.0128</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>0.6266±0.0166</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>0.5022±0.0324</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>0.4068±0.0204</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
           <t>0.6880±0.0061</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>0.6588±0.0108</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>0.5708±0.0134</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>0.4400±0.0108</t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr">
         <is>
           <t>0.6849±0.0093</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>0.7115±0.0102</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>0.7699±0.0097</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>0.8461±0.0085</t>
+        </is>
+      </c>
       <c r="N4" t="inlineStr">
         <is>
           <t>0.6636±0.0057</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>0.6594±0.0081</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>0.6268±0.0084</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>0.5533±0.0086</t>
+        </is>
+      </c>
       <c r="R4" t="inlineStr">
         <is>
           <t>0.8062±0.0049</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>0.7904±0.0055</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>0.7275±0.0102</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>0.5900±0.0088</t>
+        </is>
+      </c>
       <c r="V4" t="inlineStr">
         <is>
           <t>0.5632±0.0073</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="inlineStr"/>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>0.5526±0.0102</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>0.5030±0.0112</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>0.4088±0.0113</t>
+        </is>
+      </c>
       <c r="Z4" t="inlineStr">
         <is>
           <t>0.4326±0.0099</t>
         </is>
       </c>
-      <c r="AA4" t="inlineStr"/>
-      <c r="AB4" t="inlineStr"/>
-      <c r="AC4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>0.4438±0.0134</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>0.4545±0.0063</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>0.4422±0.0061</t>
+        </is>
+      </c>
       <c r="AD4" t="inlineStr">
         <is>
           <t>0.5465±0.0219</t>
         </is>
       </c>
-      <c r="AE4" t="inlineStr"/>
-      <c r="AF4" t="inlineStr"/>
-      <c r="AG4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>0.4709±0.0129</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>0.3896±0.0082</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>0.3394±0.0055</t>
+        </is>
+      </c>
       <c r="AH4" t="inlineStr">
         <is>
           <t>0.4332±0.0062</t>
         </is>
       </c>
-      <c r="AI4" t="inlineStr"/>
-      <c r="AJ4" t="inlineStr"/>
-      <c r="AK4" t="inlineStr"/>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>0.4659±0.0115</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>0.5543±0.0175</t>
+        </is>
+      </c>
+      <c r="AK4" t="inlineStr">
+        <is>
+          <t>0.6992±0.0134</t>
+        </is>
+      </c>
       <c r="AL4" t="inlineStr">
         <is>
           <t>1.0000±0.0000</t>
         </is>
       </c>
-      <c r="AM4" t="inlineStr"/>
-      <c r="AN4" t="inlineStr"/>
-      <c r="AO4" t="inlineStr"/>
+      <c r="AM4" t="inlineStr">
+        <is>
+          <t>0.9997±0.0008</t>
+        </is>
+      </c>
+      <c r="AN4" t="inlineStr">
+        <is>
+          <t>0.9981±0.0028</t>
+        </is>
+      </c>
+      <c r="AO4" t="inlineStr">
+        <is>
+          <t>0.9934±0.0061</t>
+        </is>
+      </c>
       <c r="AP4" t="inlineStr">
         <is>
           <t>0.6784±0.0067</t>
         </is>
       </c>
-      <c r="AQ4" t="inlineStr"/>
-      <c r="AR4" t="inlineStr"/>
-      <c r="AS4" t="inlineStr"/>
+      <c r="AQ4" t="inlineStr">
+        <is>
+          <t>0.6696±0.0086</t>
+        </is>
+      </c>
+      <c r="AR4" t="inlineStr">
+        <is>
+          <t>0.6292±0.0089</t>
+        </is>
+      </c>
+      <c r="AS4" t="inlineStr">
+        <is>
+          <t>0.5531±0.0061</t>
+        </is>
+      </c>
       <c r="AT4" t="inlineStr">
         <is>
           <t>0.6815±0.0076</t>
         </is>
       </c>
-      <c r="AU4" t="inlineStr"/>
-      <c r="AV4" t="inlineStr"/>
-      <c r="AW4" t="inlineStr"/>
+      <c r="AU4" t="inlineStr">
+        <is>
+          <t>0.6402±0.0102</t>
+        </is>
+      </c>
+      <c r="AV4" t="inlineStr">
+        <is>
+          <t>0.5353±0.0134</t>
+        </is>
+      </c>
+      <c r="AW4" t="inlineStr">
+        <is>
+          <t>0.4127±0.0067</t>
+        </is>
+      </c>
       <c r="AX4" t="inlineStr">
         <is>
           <t>0.6755±0.0107</t>
         </is>
       </c>
-      <c r="AY4" t="inlineStr"/>
-      <c r="AZ4" t="inlineStr"/>
-      <c r="BA4" t="inlineStr"/>
+      <c r="AY4" t="inlineStr">
+        <is>
+          <t>0.7021±0.0137</t>
+        </is>
+      </c>
+      <c r="AZ4" t="inlineStr">
+        <is>
+          <t>0.7636±0.0126</t>
+        </is>
+      </c>
+      <c r="BA4" t="inlineStr">
+        <is>
+          <t>0.8385±0.0105</t>
+        </is>
+      </c>
       <c r="BB4" t="inlineStr">
         <is>
           <t>0.2313±0.0201</t>
         </is>
       </c>
-      <c r="BC4" t="inlineStr"/>
-      <c r="BD4" t="inlineStr"/>
-      <c r="BE4" t="inlineStr"/>
+      <c r="BC4" t="inlineStr">
+        <is>
+          <t>0.1916±0.0213</t>
+        </is>
+      </c>
+      <c r="BD4" t="inlineStr">
+        <is>
+          <t>0.1022±0.0168</t>
+        </is>
+      </c>
+      <c r="BE4" t="inlineStr">
+        <is>
+          <t>0.0226±0.0135</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1083,113 +1587,281 @@
           <t>0.6610±0.0104</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>0.6292±0.0164</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>0.5053±0.0316</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>0.4133±0.0205</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>0.6788±0.0081</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>0.6507±0.0108</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>0.5652±0.0140</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>0.4366±0.0102</t>
+        </is>
+      </c>
       <c r="J5" t="inlineStr">
         <is>
           <t>0.7093±0.0104</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>0.7241±0.0106</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>0.7789±0.0082</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>0.8501±0.0084</t>
+        </is>
+      </c>
       <c r="N5" t="inlineStr">
         <is>
           <t>0.6709±0.0062</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>0.6612±0.0084</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>0.6271±0.0090</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>0.5523±0.0083</t>
+        </is>
+      </c>
       <c r="R5" t="inlineStr">
         <is>
           <t>0.8048±0.0055</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>0.7879±0.0058</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>0.7253±0.0107</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>0.5877±0.0091</t>
+        </is>
+      </c>
       <c r="V5" t="inlineStr">
         <is>
           <t>0.5695±0.0072</t>
         </is>
       </c>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
-      <c r="Y5" t="inlineStr"/>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>0.5533±0.0104</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>0.5021±0.0118</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>0.4068±0.0105</t>
+        </is>
+      </c>
       <c r="Z5" t="inlineStr">
         <is>
           <t>0.4417±0.0089</t>
         </is>
       </c>
-      <c r="AA5" t="inlineStr"/>
-      <c r="AB5" t="inlineStr"/>
-      <c r="AC5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>0.4481±0.0126</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>0.4567±0.0073</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>0.4424±0.0063</t>
+        </is>
+      </c>
       <c r="AD5" t="inlineStr">
         <is>
           <t>0.5408±0.0179</t>
         </is>
       </c>
-      <c r="AE5" t="inlineStr"/>
-      <c r="AF5" t="inlineStr"/>
-      <c r="AG5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>0.4683±0.0097</t>
+        </is>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>0.3885±0.0088</t>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>0.3388±0.0056</t>
+        </is>
+      </c>
       <c r="AH5" t="inlineStr">
         <is>
           <t>0.4532±0.0068</t>
         </is>
       </c>
-      <c r="AI5" t="inlineStr"/>
-      <c r="AJ5" t="inlineStr"/>
-      <c r="AK5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr">
+        <is>
+          <t>0.4781±0.0109</t>
+        </is>
+      </c>
+      <c r="AJ5" t="inlineStr">
+        <is>
+          <t>0.5636±0.0171</t>
+        </is>
+      </c>
+      <c r="AK5" t="inlineStr">
+        <is>
+          <t>0.7035±0.0147</t>
+        </is>
+      </c>
       <c r="AL5" t="inlineStr">
         <is>
           <t>1.0000±0.0000</t>
         </is>
       </c>
-      <c r="AM5" t="inlineStr"/>
-      <c r="AN5" t="inlineStr"/>
-      <c r="AO5" t="inlineStr"/>
+      <c r="AM5" t="inlineStr">
+        <is>
+          <t>1.0000±0.0000</t>
+        </is>
+      </c>
+      <c r="AN5" t="inlineStr">
+        <is>
+          <t>0.9989±0.0025</t>
+        </is>
+      </c>
+      <c r="AO5" t="inlineStr">
+        <is>
+          <t>0.9942±0.0060</t>
+        </is>
+      </c>
       <c r="AP5" t="inlineStr">
         <is>
           <t>0.6840±0.0074</t>
         </is>
       </c>
-      <c r="AQ5" t="inlineStr"/>
-      <c r="AR5" t="inlineStr"/>
-      <c r="AS5" t="inlineStr"/>
+      <c r="AQ5" t="inlineStr">
+        <is>
+          <t>0.6711±0.0085</t>
+        </is>
+      </c>
+      <c r="AR5" t="inlineStr">
+        <is>
+          <t>0.6300±0.0095</t>
+        </is>
+      </c>
+      <c r="AS5" t="inlineStr">
+        <is>
+          <t>0.5530±0.0061</t>
+        </is>
+      </c>
       <c r="AT5" t="inlineStr">
         <is>
           <t>0.6707±0.0093</t>
         </is>
       </c>
-      <c r="AU5" t="inlineStr"/>
-      <c r="AV5" t="inlineStr"/>
-      <c r="AW5" t="inlineStr"/>
+      <c r="AU5" t="inlineStr">
+        <is>
+          <t>0.6324±0.0095</t>
+        </is>
+      </c>
+      <c r="AV5" t="inlineStr">
+        <is>
+          <t>0.5321±0.0138</t>
+        </is>
+      </c>
+      <c r="AW5" t="inlineStr">
+        <is>
+          <t>0.4116±0.0067</t>
+        </is>
+      </c>
       <c r="AX5" t="inlineStr">
         <is>
           <t>0.6979±0.0113</t>
         </is>
       </c>
-      <c r="AY5" t="inlineStr"/>
-      <c r="AZ5" t="inlineStr"/>
-      <c r="BA5" t="inlineStr"/>
+      <c r="AY5" t="inlineStr">
+        <is>
+          <t>0.7150±0.0131</t>
+        </is>
+      </c>
+      <c r="AZ5" t="inlineStr">
+        <is>
+          <t>0.7727±0.0110</t>
+        </is>
+      </c>
+      <c r="BA5" t="inlineStr">
+        <is>
+          <t>0.8428±0.0104</t>
+        </is>
+      </c>
       <c r="BB5" t="inlineStr">
         <is>
           <t>0.2242±0.0196</t>
         </is>
       </c>
-      <c r="BC5" t="inlineStr"/>
-      <c r="BD5" t="inlineStr"/>
-      <c r="BE5" t="inlineStr"/>
+      <c r="BC5" t="inlineStr">
+        <is>
+          <t>0.1791±0.0184</t>
+        </is>
+      </c>
+      <c r="BD5" t="inlineStr">
+        <is>
+          <t>0.0923±0.0146</t>
+        </is>
+      </c>
+      <c r="BE5" t="inlineStr">
+        <is>
+          <t>0.0155±0.0093</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1202,113 +1874,281 @@
           <t>0.7456±0.0120</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>0.7434±0.0117</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>0.7311±0.0159</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0.6613±0.0155</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
           <t>0.7328±0.0084</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>0.7276±0.0084</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>0.7103±0.0094</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>0.6613±0.0110</t>
+        </is>
+      </c>
       <c r="J6" t="inlineStr">
         <is>
           <t>0.6002±0.0129</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>0.6003±0.0119</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>0.6015±0.0162</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>0.6211±0.0102</t>
+        </is>
+      </c>
       <c r="N6" t="inlineStr">
         <is>
           <t>0.6319±0.0076</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>0.6304±0.0075</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>0.6246±0.0079</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>0.6158±0.0059</t>
+        </is>
+      </c>
       <c r="R6" t="inlineStr">
         <is>
           <t>0.8129±0.0040</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>0.8102±0.0041</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>0.8033±0.0047</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>0.7836±0.0058</t>
+        </is>
+      </c>
       <c r="V6" t="inlineStr">
         <is>
           <t>0.5295±0.0075</t>
         </is>
       </c>
-      <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr"/>
-      <c r="Y6" t="inlineStr"/>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>0.5258±0.0092</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>0.5169±0.0098</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>0.4996±0.0096</t>
+        </is>
+      </c>
       <c r="Z6" t="inlineStr">
         <is>
           <t>0.3791±0.0081</t>
         </is>
       </c>
-      <c r="AA6" t="inlineStr"/>
-      <c r="AB6" t="inlineStr"/>
-      <c r="AC6" t="inlineStr"/>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>0.3739±0.0089</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>0.3735±0.0107</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>0.3894±0.0063</t>
+        </is>
+      </c>
       <c r="AD6" t="inlineStr">
         <is>
           <t>0.6452±0.0624</t>
         </is>
       </c>
-      <c r="AE6" t="inlineStr"/>
-      <c r="AF6" t="inlineStr"/>
-      <c r="AG6" t="inlineStr"/>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>0.6215±0.0547</t>
+        </is>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>0.5549±0.0493</t>
+        </is>
+      </c>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>0.4592±0.0262</t>
+        </is>
+      </c>
       <c r="AH6" t="inlineStr">
         <is>
           <t>0.3516±0.0080</t>
         </is>
       </c>
-      <c r="AI6" t="inlineStr"/>
-      <c r="AJ6" t="inlineStr"/>
-      <c r="AK6" t="inlineStr"/>
+      <c r="AI6" t="inlineStr">
+        <is>
+          <t>0.3501±0.0084</t>
+        </is>
+      </c>
+      <c r="AJ6" t="inlineStr">
+        <is>
+          <t>0.3530±0.0125</t>
+        </is>
+      </c>
+      <c r="AK6" t="inlineStr">
+        <is>
+          <t>0.3828±0.0072</t>
+        </is>
+      </c>
       <c r="AL6" t="inlineStr">
         <is>
           <t>1.0000±0.0000</t>
         </is>
       </c>
-      <c r="AM6" t="inlineStr"/>
-      <c r="AN6" t="inlineStr"/>
-      <c r="AO6" t="inlineStr"/>
+      <c r="AM6" t="inlineStr">
+        <is>
+          <t>1.0000±0.0000</t>
+        </is>
+      </c>
+      <c r="AN6" t="inlineStr">
+        <is>
+          <t>0.9998±0.0006</t>
+        </is>
+      </c>
+      <c r="AO6" t="inlineStr">
+        <is>
+          <t>0.9929±0.0037</t>
+        </is>
+      </c>
       <c r="AP6" t="inlineStr">
         <is>
           <t>0.6573±0.0072</t>
         </is>
       </c>
-      <c r="AQ6" t="inlineStr"/>
-      <c r="AR6" t="inlineStr"/>
-      <c r="AS6" t="inlineStr"/>
+      <c r="AQ6" t="inlineStr">
+        <is>
+          <t>0.6538±0.0078</t>
+        </is>
+      </c>
+      <c r="AR6" t="inlineStr">
+        <is>
+          <t>0.6458±0.0087</t>
+        </is>
+      </c>
+      <c r="AS6" t="inlineStr">
+        <is>
+          <t>0.6318±0.0069</t>
+        </is>
+      </c>
       <c r="AT6" t="inlineStr">
         <is>
           <t>0.7376±0.0078</t>
         </is>
       </c>
-      <c r="AU6" t="inlineStr"/>
-      <c r="AV6" t="inlineStr"/>
-      <c r="AW6" t="inlineStr"/>
+      <c r="AU6" t="inlineStr">
+        <is>
+          <t>0.7296±0.0081</t>
+        </is>
+      </c>
+      <c r="AV6" t="inlineStr">
+        <is>
+          <t>0.7101±0.0102</t>
+        </is>
+      </c>
+      <c r="AW6" t="inlineStr">
+        <is>
+          <t>0.6516±0.0109</t>
+        </is>
+      </c>
       <c r="AX6" t="inlineStr">
         <is>
           <t>0.5930±0.0132</t>
         </is>
       </c>
-      <c r="AY6" t="inlineStr"/>
-      <c r="AZ6" t="inlineStr"/>
-      <c r="BA6" t="inlineStr"/>
+      <c r="AY6" t="inlineStr">
+        <is>
+          <t>0.5924±0.0131</t>
+        </is>
+      </c>
+      <c r="AZ6" t="inlineStr">
+        <is>
+          <t>0.5926±0.0173</t>
+        </is>
+      </c>
+      <c r="BA6" t="inlineStr">
+        <is>
+          <t>0.6135±0.0121</t>
+        </is>
+      </c>
       <c r="BB6" t="inlineStr">
         <is>
           <t>0.2003±0.0158</t>
         </is>
       </c>
-      <c r="BC6" t="inlineStr"/>
-      <c r="BD6" t="inlineStr"/>
-      <c r="BE6" t="inlineStr"/>
+      <c r="BC6" t="inlineStr">
+        <is>
+          <t>0.1891±0.0221</t>
+        </is>
+      </c>
+      <c r="BD6" t="inlineStr">
+        <is>
+          <t>0.1647±0.0277</t>
+        </is>
+      </c>
+      <c r="BE6" t="inlineStr">
+        <is>
+          <t>0.1227±0.0257</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1321,113 +2161,281 @@
           <t>0.6897±0.0141</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>0.6740±0.0177</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>0.6317±0.0205</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>0.5345±0.0390</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>0.6763±0.0083</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>0.6592±0.0121</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>0.6149±0.0133</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>0.5197±0.0124</t>
+        </is>
+      </c>
       <c r="J7" t="inlineStr">
         <is>
           <t>0.7002±0.0115</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>0.7149±0.0100</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>0.7430±0.0118</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>0.7849±0.0111</t>
+        </is>
+      </c>
       <c r="N7" t="inlineStr">
         <is>
           <t>0.6662±0.0051</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>0.6635±0.0082</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>0.6501±0.0089</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>0.6031±0.0088</t>
+        </is>
+      </c>
       <c r="R7" t="inlineStr">
         <is>
           <t>0.8042±0.0049</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>0.7964±0.0066</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>0.7733±0.0073</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>0.7043±0.0092</t>
+        </is>
+      </c>
       <c r="V7" t="inlineStr">
         <is>
           <t>0.5633±0.0057</t>
         </is>
       </c>
-      <c r="W7" t="inlineStr"/>
-      <c r="X7" t="inlineStr"/>
-      <c r="Y7" t="inlineStr"/>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>0.5557±0.0103</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>0.5326±0.0099</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>0.4653±0.0103</t>
+        </is>
+      </c>
       <c r="Z7" t="inlineStr">
         <is>
           <t>0.4256±0.0092</t>
         </is>
       </c>
-      <c r="AA7" t="inlineStr"/>
-      <c r="AB7" t="inlineStr"/>
-      <c r="AC7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>0.4296±0.0131</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>0.4389±0.0088</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>0.4403±0.0115</t>
+        </is>
+      </c>
       <c r="AD7" t="inlineStr">
         <is>
           <t>0.5841±0.0319</t>
         </is>
       </c>
-      <c r="AE7" t="inlineStr"/>
-      <c r="AF7" t="inlineStr"/>
-      <c r="AG7" t="inlineStr"/>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>0.5255±0.0245</t>
+        </is>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>0.4418±0.0168</t>
+        </is>
+      </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>0.3666±0.0104</t>
+        </is>
+      </c>
       <c r="AH7" t="inlineStr">
         <is>
           <t>0.4380±0.0091</t>
         </is>
       </c>
-      <c r="AI7" t="inlineStr"/>
-      <c r="AJ7" t="inlineStr"/>
-      <c r="AK7" t="inlineStr"/>
+      <c r="AI7" t="inlineStr">
+        <is>
+          <t>0.4544±0.0086</t>
+        </is>
+      </c>
+      <c r="AJ7" t="inlineStr">
+        <is>
+          <t>0.4912±0.0073</t>
+        </is>
+      </c>
+      <c r="AK7" t="inlineStr">
+        <is>
+          <t>0.5643±0.0172</t>
+        </is>
+      </c>
       <c r="AL7" t="inlineStr">
         <is>
           <t>1.0000±0.0000</t>
         </is>
       </c>
-      <c r="AM7" t="inlineStr"/>
-      <c r="AN7" t="inlineStr"/>
-      <c r="AO7" t="inlineStr"/>
+      <c r="AM7" t="inlineStr">
+        <is>
+          <t>1.0000±0.0000</t>
+        </is>
+      </c>
+      <c r="AN7" t="inlineStr">
+        <is>
+          <t>0.9997±0.0008</t>
+        </is>
+      </c>
+      <c r="AO7" t="inlineStr">
+        <is>
+          <t>0.9964±0.0047</t>
+        </is>
+      </c>
       <c r="AP7" t="inlineStr">
         <is>
           <t>0.6804±0.0060</t>
         </is>
       </c>
-      <c r="AQ7" t="inlineStr"/>
-      <c r="AR7" t="inlineStr"/>
-      <c r="AS7" t="inlineStr"/>
+      <c r="AQ7" t="inlineStr">
+        <is>
+          <t>0.6766±0.0085</t>
+        </is>
+      </c>
+      <c r="AR7" t="inlineStr">
+        <is>
+          <t>0.6617±0.0086</t>
+        </is>
+      </c>
+      <c r="AS7" t="inlineStr">
+        <is>
+          <t>0.6140±0.0083</t>
+        </is>
+      </c>
       <c r="AT7" t="inlineStr">
         <is>
           <t>0.6724±0.0091</t>
         </is>
       </c>
-      <c r="AU7" t="inlineStr"/>
-      <c r="AV7" t="inlineStr"/>
-      <c r="AW7" t="inlineStr"/>
+      <c r="AU7" t="inlineStr">
+        <is>
+          <t>0.6517±0.0118</t>
+        </is>
+      </c>
+      <c r="AV7" t="inlineStr">
+        <is>
+          <t>0.6036±0.0129</t>
+        </is>
+      </c>
+      <c r="AW7" t="inlineStr">
+        <is>
+          <t>0.5077±0.0106</t>
+        </is>
+      </c>
       <c r="AX7" t="inlineStr">
         <is>
           <t>0.6889±0.0115</t>
         </is>
       </c>
-      <c r="AY7" t="inlineStr"/>
-      <c r="AZ7" t="inlineStr"/>
-      <c r="BA7" t="inlineStr"/>
+      <c r="AY7" t="inlineStr">
+        <is>
+          <t>0.7036±0.0111</t>
+        </is>
+      </c>
+      <c r="AZ7" t="inlineStr">
+        <is>
+          <t>0.7324±0.0104</t>
+        </is>
+      </c>
+      <c r="BA7" t="inlineStr">
+        <is>
+          <t>0.7770±0.0121</t>
+        </is>
+      </c>
       <c r="BB7" t="inlineStr">
         <is>
           <t>0.2122±0.0188</t>
         </is>
       </c>
-      <c r="BC7" t="inlineStr"/>
-      <c r="BD7" t="inlineStr"/>
-      <c r="BE7" t="inlineStr"/>
+      <c r="BC7" t="inlineStr">
+        <is>
+          <t>0.1771±0.0226</t>
+        </is>
+      </c>
+      <c r="BD7" t="inlineStr">
+        <is>
+          <t>0.1084±0.0144</t>
+        </is>
+      </c>
+      <c r="BE7" t="inlineStr">
+        <is>
+          <t>0.0199±0.0095</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1440,113 +2448,281 @@
           <t>0.7758±0.0119</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>0.7706±0.0111</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>0.7542±0.0157</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>0.6752±0.0149</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
           <t>0.7404±0.0067</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0.7346±0.0063</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>0.7190±0.0098</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>0.6654±0.0109</t>
+        </is>
+      </c>
       <c r="J8" t="inlineStr">
         <is>
           <t>0.5714±0.0146</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>0.5733±0.0122</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>0.5788±0.0146</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>0.6007±0.0103</t>
+        </is>
+      </c>
       <c r="N8" t="inlineStr">
         <is>
           <t>0.6163±0.0091</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>0.6161±0.0081</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>0.6140±0.0072</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>0.6061±0.0066</t>
+        </is>
+      </c>
       <c r="R8" t="inlineStr">
         <is>
           <t>0.8101±0.0044</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr"/>
-      <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr"/>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>0.8079±0.0045</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>0.8023±0.0043</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>0.7821±0.0058</t>
+        </is>
+      </c>
       <c r="V8" t="inlineStr">
         <is>
           <t>0.5126±0.0095</t>
         </is>
       </c>
-      <c r="W8" t="inlineStr"/>
-      <c r="X8" t="inlineStr"/>
-      <c r="Y8" t="inlineStr"/>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>0.5097±0.0095</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>0.5049±0.0086</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>0.4891±0.0105</t>
+        </is>
+      </c>
       <c r="Z8" t="inlineStr">
         <is>
           <t>0.3604±0.0093</t>
         </is>
       </c>
-      <c r="AA8" t="inlineStr"/>
-      <c r="AB8" t="inlineStr"/>
-      <c r="AC8" t="inlineStr"/>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>0.3582±0.0102</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>0.3605±0.0094</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>0.3784±0.0068</t>
+        </is>
+      </c>
       <c r="AD8" t="inlineStr">
         <is>
           <t>0.6261±0.0679</t>
         </is>
       </c>
-      <c r="AE8" t="inlineStr"/>
-      <c r="AF8" t="inlineStr"/>
-      <c r="AG8" t="inlineStr"/>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>0.6292±0.0570</t>
+        </is>
+      </c>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>0.5549±0.0490</t>
+        </is>
+      </c>
+      <c r="AG8" t="inlineStr">
+        <is>
+          <t>0.4554±0.0235</t>
+        </is>
+      </c>
       <c r="AH8" t="inlineStr">
         <is>
           <t>0.3289±0.0085</t>
         </is>
       </c>
-      <c r="AI8" t="inlineStr"/>
-      <c r="AJ8" t="inlineStr"/>
-      <c r="AK8" t="inlineStr"/>
+      <c r="AI8" t="inlineStr">
+        <is>
+          <t>0.3290±0.0084</t>
+        </is>
+      </c>
+      <c r="AJ8" t="inlineStr">
+        <is>
+          <t>0.3346±0.0109</t>
+        </is>
+      </c>
+      <c r="AK8" t="inlineStr">
+        <is>
+          <t>0.3659±0.0077</t>
+        </is>
+      </c>
       <c r="AL8" t="inlineStr">
         <is>
           <t>1.0000±0.0000</t>
         </is>
       </c>
-      <c r="AM8" t="inlineStr"/>
-      <c r="AN8" t="inlineStr"/>
-      <c r="AO8" t="inlineStr"/>
+      <c r="AM8" t="inlineStr">
+        <is>
+          <t>1.0000±0.0000</t>
+        </is>
+      </c>
+      <c r="AN8" t="inlineStr">
+        <is>
+          <t>0.9998±0.0006</t>
+        </is>
+      </c>
+      <c r="AO8" t="inlineStr">
+        <is>
+          <t>0.9919±0.0033</t>
+        </is>
+      </c>
       <c r="AP8" t="inlineStr">
         <is>
           <t>0.6437±0.0084</t>
         </is>
       </c>
-      <c r="AQ8" t="inlineStr"/>
-      <c r="AR8" t="inlineStr"/>
-      <c r="AS8" t="inlineStr"/>
+      <c r="AQ8" t="inlineStr">
+        <is>
+          <t>0.6411±0.0083</t>
+        </is>
+      </c>
+      <c r="AR8" t="inlineStr">
+        <is>
+          <t>0.6358±0.0080</t>
+        </is>
+      </c>
+      <c r="AS8" t="inlineStr">
+        <is>
+          <t>0.6224±0.0074</t>
+        </is>
+      </c>
       <c r="AT8" t="inlineStr">
         <is>
           <t>0.7449±0.0060</t>
         </is>
       </c>
-      <c r="AU8" t="inlineStr"/>
-      <c r="AV8" t="inlineStr"/>
-      <c r="AW8" t="inlineStr"/>
+      <c r="AU8" t="inlineStr">
+        <is>
+          <t>0.7376±0.0061</t>
+        </is>
+      </c>
+      <c r="AV8" t="inlineStr">
+        <is>
+          <t>0.7186±0.0106</t>
+        </is>
+      </c>
+      <c r="AW8" t="inlineStr">
+        <is>
+          <t>0.6546±0.0110</t>
+        </is>
+      </c>
       <c r="AX8" t="inlineStr">
         <is>
           <t>0.5669±0.0142</t>
         </is>
       </c>
-      <c r="AY8" t="inlineStr"/>
-      <c r="AZ8" t="inlineStr"/>
-      <c r="BA8" t="inlineStr"/>
+      <c r="AY8" t="inlineStr">
+        <is>
+          <t>0.5670±0.0130</t>
+        </is>
+      </c>
+      <c r="AZ8" t="inlineStr">
+        <is>
+          <t>0.5706±0.0153</t>
+        </is>
+      </c>
+      <c r="BA8" t="inlineStr">
+        <is>
+          <t>0.5934±0.0122</t>
+        </is>
+      </c>
       <c r="BB8" t="inlineStr">
         <is>
           <t>0.1796±0.0146</t>
         </is>
       </c>
-      <c r="BC8" t="inlineStr"/>
-      <c r="BD8" t="inlineStr"/>
-      <c r="BE8" t="inlineStr"/>
+      <c r="BC8" t="inlineStr">
+        <is>
+          <t>0.1645±0.0197</t>
+        </is>
+      </c>
+      <c r="BD8" t="inlineStr">
+        <is>
+          <t>0.1485±0.0233</t>
+        </is>
+      </c>
+      <c r="BE8" t="inlineStr">
+        <is>
+          <t>0.1146±0.0276</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1559,113 +2735,281 @@
           <t>0.6898±0.0158</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>0.6744±0.0184</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>0.6309±0.0193</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>0.5322±0.0423</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
           <t>0.6773±0.0082</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>0.6592±0.0122</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>0.6152±0.0126</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>0.5192±0.0122</t>
+        </is>
+      </c>
       <c r="J9" t="inlineStr">
         <is>
           <t>0.6993±0.0121</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>0.7142±0.0101</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>0.7431±0.0113</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>0.7838±0.0114</t>
+        </is>
+      </c>
       <c r="N9" t="inlineStr">
         <is>
           <t>0.6664±0.0054</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>0.6631±0.0085</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>0.6504±0.0085</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>0.6025±0.0089</t>
+        </is>
+      </c>
       <c r="R9" t="inlineStr">
         <is>
           <t>0.8047±0.0050</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr"/>
-      <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr"/>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>0.7964±0.0069</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>0.7736±0.0072</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>0.7040±0.0089</t>
+        </is>
+      </c>
       <c r="V9" t="inlineStr">
         <is>
           <t>0.5635±0.0059</t>
         </is>
       </c>
-      <c r="W9" t="inlineStr"/>
-      <c r="X9" t="inlineStr"/>
-      <c r="Y9" t="inlineStr"/>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>0.5553±0.0104</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>0.5331±0.0093</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>0.4647±0.0103</t>
+        </is>
+      </c>
       <c r="Z9" t="inlineStr">
         <is>
           <t>0.4267±0.0097</t>
         </is>
       </c>
-      <c r="AA9" t="inlineStr"/>
-      <c r="AB9" t="inlineStr"/>
-      <c r="AC9" t="inlineStr"/>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>0.4288±0.0128</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>0.4398±0.0072</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>0.4402±0.0121</t>
+        </is>
+      </c>
       <c r="AD9" t="inlineStr">
         <is>
           <t>0.5870±0.0326</t>
         </is>
       </c>
-      <c r="AE9" t="inlineStr"/>
-      <c r="AF9" t="inlineStr"/>
-      <c r="AG9" t="inlineStr"/>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>0.5282±0.0258</t>
+        </is>
+      </c>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>0.4455±0.0141</t>
+        </is>
+      </c>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>0.3663±0.0104</t>
+        </is>
+      </c>
       <c r="AH9" t="inlineStr">
         <is>
           <t>0.4379±0.0094</t>
         </is>
       </c>
-      <c r="AI9" t="inlineStr"/>
-      <c r="AJ9" t="inlineStr"/>
-      <c r="AK9" t="inlineStr"/>
+      <c r="AI9" t="inlineStr">
+        <is>
+          <t>0.4535±0.0083</t>
+        </is>
+      </c>
+      <c r="AJ9" t="inlineStr">
+        <is>
+          <t>0.4916±0.0074</t>
+        </is>
+      </c>
+      <c r="AK9" t="inlineStr">
+        <is>
+          <t>0.5643±0.0178</t>
+        </is>
+      </c>
       <c r="AL9" t="inlineStr">
         <is>
           <t>1.0000±0.0000</t>
         </is>
       </c>
-      <c r="AM9" t="inlineStr"/>
-      <c r="AN9" t="inlineStr"/>
-      <c r="AO9" t="inlineStr"/>
+      <c r="AM9" t="inlineStr">
+        <is>
+          <t>1.0000±0.0000</t>
+        </is>
+      </c>
+      <c r="AN9" t="inlineStr">
+        <is>
+          <t>0.9997±0.0008</t>
+        </is>
+      </c>
+      <c r="AO9" t="inlineStr">
+        <is>
+          <t>0.9964±0.0047</t>
+        </is>
+      </c>
       <c r="AP9" t="inlineStr">
         <is>
           <t>0.6808±0.0061</t>
         </is>
       </c>
-      <c r="AQ9" t="inlineStr"/>
-      <c r="AR9" t="inlineStr"/>
-      <c r="AS9" t="inlineStr"/>
+      <c r="AQ9" t="inlineStr">
+        <is>
+          <t>0.6763±0.0089</t>
+        </is>
+      </c>
+      <c r="AR9" t="inlineStr">
+        <is>
+          <t>0.6620±0.0082</t>
+        </is>
+      </c>
+      <c r="AS9" t="inlineStr">
+        <is>
+          <t>0.6136±0.0085</t>
+        </is>
+      </c>
       <c r="AT9" t="inlineStr">
         <is>
           <t>0.6738±0.0089</t>
         </is>
       </c>
-      <c r="AU9" t="inlineStr"/>
-      <c r="AV9" t="inlineStr"/>
-      <c r="AW9" t="inlineStr"/>
+      <c r="AU9" t="inlineStr">
+        <is>
+          <t>0.6518±0.0119</t>
+        </is>
+      </c>
+      <c r="AV9" t="inlineStr">
+        <is>
+          <t>0.6040±0.0121</t>
+        </is>
+      </c>
+      <c r="AW9" t="inlineStr">
+        <is>
+          <t>0.5074±0.0105</t>
+        </is>
+      </c>
       <c r="AX9" t="inlineStr">
         <is>
           <t>0.6882±0.0116</t>
         </is>
       </c>
-      <c r="AY9" t="inlineStr"/>
-      <c r="AZ9" t="inlineStr"/>
-      <c r="BA9" t="inlineStr"/>
+      <c r="AY9" t="inlineStr">
+        <is>
+          <t>0.7029±0.0111</t>
+        </is>
+      </c>
+      <c r="AZ9" t="inlineStr">
+        <is>
+          <t>0.7325±0.0105</t>
+        </is>
+      </c>
+      <c r="BA9" t="inlineStr">
+        <is>
+          <t>0.7762±0.0129</t>
+        </is>
+      </c>
       <c r="BB9" t="inlineStr">
         <is>
           <t>0.2127±0.0204</t>
         </is>
       </c>
-      <c r="BC9" t="inlineStr"/>
-      <c r="BD9" t="inlineStr"/>
-      <c r="BE9" t="inlineStr"/>
+      <c r="BC9" t="inlineStr">
+        <is>
+          <t>0.1761±0.0221</t>
+        </is>
+      </c>
+      <c r="BD9" t="inlineStr">
+        <is>
+          <t>0.1084±0.0131</t>
+        </is>
+      </c>
+      <c r="BE9" t="inlineStr">
+        <is>
+          <t>0.0186±0.0096</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1678,113 +3022,281 @@
           <t>0.7799±0.0118</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>0.7738±0.0153</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>0.7496±0.0202</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>0.6818±0.0135</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
           <t>0.7393±0.0078</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>0.7313±0.0096</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>0.7112±0.0085</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>0.6628±0.0115</t>
+        </is>
+      </c>
       <c r="J10" t="inlineStr">
         <is>
           <t>0.5636±0.0121</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>0.5589±0.0140</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>0.5504±0.0122</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>0.5310±0.0141</t>
+        </is>
+      </c>
       <c r="N10" t="inlineStr">
         <is>
           <t>0.6093±0.0074</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>0.6047±0.0086</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>0.5913±0.0060</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>0.5577±0.0092</t>
+        </is>
+      </c>
       <c r="R10" t="inlineStr">
         <is>
           <t>0.8091±0.0040</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr"/>
-      <c r="T10" t="inlineStr"/>
-      <c r="U10" t="inlineStr"/>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>0.8059±0.0048</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>0.7975±0.0030</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>0.7746±0.0032</t>
+        </is>
+      </c>
       <c r="V10" t="inlineStr">
         <is>
           <t>0.5035±0.0095</t>
         </is>
       </c>
-      <c r="W10" t="inlineStr"/>
-      <c r="X10" t="inlineStr"/>
-      <c r="Y10" t="inlineStr"/>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>0.4966±0.0094</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>0.4803±0.0055</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>0.4393±0.0090</t>
+        </is>
+      </c>
       <c r="Z10" t="inlineStr">
         <is>
           <t>0.3626±0.0080</t>
         </is>
       </c>
-      <c r="AA10" t="inlineStr"/>
-      <c r="AB10" t="inlineStr"/>
-      <c r="AC10" t="inlineStr"/>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>0.3573±0.0107</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>0.3561±0.0104</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>0.3602±0.0105</t>
+        </is>
+      </c>
       <c r="AD10" t="inlineStr">
         <is>
           <t>0.6401±0.0548</t>
         </is>
       </c>
-      <c r="AE10" t="inlineStr"/>
-      <c r="AF10" t="inlineStr"/>
-      <c r="AG10" t="inlineStr"/>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>0.6218±0.0528</t>
+        </is>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>0.5597±0.0264</t>
+        </is>
+      </c>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>0.4618±0.0220</t>
+        </is>
+      </c>
       <c r="AH10" t="inlineStr">
         <is>
           <t>0.3247±0.0081</t>
         </is>
       </c>
-      <c r="AI10" t="inlineStr"/>
-      <c r="AJ10" t="inlineStr"/>
-      <c r="AK10" t="inlineStr"/>
+      <c r="AI10" t="inlineStr">
+        <is>
+          <t>0.3222±0.0105</t>
+        </is>
+      </c>
+      <c r="AJ10" t="inlineStr">
+        <is>
+          <t>0.3217±0.0115</t>
+        </is>
+      </c>
+      <c r="AK10" t="inlineStr">
+        <is>
+          <t>0.3265±0.0095</t>
+        </is>
+      </c>
       <c r="AL10" t="inlineStr">
         <is>
           <t>1.0000±0.0000</t>
         </is>
       </c>
-      <c r="AM10" t="inlineStr"/>
-      <c r="AN10" t="inlineStr"/>
-      <c r="AO10" t="inlineStr"/>
+      <c r="AM10" t="inlineStr">
+        <is>
+          <t>1.0000±0.0000</t>
+        </is>
+      </c>
+      <c r="AN10" t="inlineStr">
+        <is>
+          <t>0.9998±0.0006</t>
+        </is>
+      </c>
+      <c r="AO10" t="inlineStr">
+        <is>
+          <t>0.9945±0.0035</t>
+        </is>
+      </c>
       <c r="AP10" t="inlineStr">
         <is>
           <t>0.6392±0.0077</t>
         </is>
       </c>
-      <c r="AQ10" t="inlineStr"/>
-      <c r="AR10" t="inlineStr"/>
-      <c r="AS10" t="inlineStr"/>
+      <c r="AQ10" t="inlineStr">
+        <is>
+          <t>0.6340±0.0085</t>
+        </is>
+      </c>
+      <c r="AR10" t="inlineStr">
+        <is>
+          <t>0.6203±0.0051</t>
+        </is>
+      </c>
+      <c r="AS10" t="inlineStr">
+        <is>
+          <t>0.5859±0.0077</t>
+        </is>
+      </c>
       <c r="AT10" t="inlineStr">
         <is>
           <t>0.7469±0.0085</t>
         </is>
       </c>
-      <c r="AU10" t="inlineStr"/>
-      <c r="AV10" t="inlineStr"/>
-      <c r="AW10" t="inlineStr"/>
+      <c r="AU10" t="inlineStr">
+        <is>
+          <t>0.7385±0.0107</t>
+        </is>
+      </c>
+      <c r="AV10" t="inlineStr">
+        <is>
+          <t>0.7172±0.0111</t>
+        </is>
+      </c>
+      <c r="AW10" t="inlineStr">
+        <is>
+          <t>0.6599±0.0132</t>
+        </is>
+      </c>
       <c r="AX10" t="inlineStr">
         <is>
           <t>0.5589±0.0129</t>
         </is>
       </c>
-      <c r="AY10" t="inlineStr"/>
-      <c r="AZ10" t="inlineStr"/>
-      <c r="BA10" t="inlineStr"/>
+      <c r="AY10" t="inlineStr">
+        <is>
+          <t>0.5557±0.0146</t>
+        </is>
+      </c>
+      <c r="AZ10" t="inlineStr">
+        <is>
+          <t>0.5468±0.0128</t>
+        </is>
+      </c>
+      <c r="BA10" t="inlineStr">
+        <is>
+          <t>0.5271±0.0126</t>
+        </is>
+      </c>
       <c r="BB10" t="inlineStr">
         <is>
           <t>0.1667±0.0175</t>
         </is>
       </c>
-      <c r="BC10" t="inlineStr"/>
-      <c r="BD10" t="inlineStr"/>
-      <c r="BE10" t="inlineStr"/>
+      <c r="BC10" t="inlineStr">
+        <is>
+          <t>0.1506±0.0133</t>
+        </is>
+      </c>
+      <c r="BD10" t="inlineStr">
+        <is>
+          <t>0.1254±0.0115</t>
+        </is>
+      </c>
+      <c r="BE10" t="inlineStr">
+        <is>
+          <t>0.0782±0.0120</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1797,113 +3309,281 @@
           <t>0.7515±0.0154</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>0.7705±0.0141</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>0.7577±0.0057</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>0.6870±0.0191</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr">
         <is>
           <t>0.7275±0.0083</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>0.7327±0.0091</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>0.7184±0.0109</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>0.6629±0.0149</t>
+        </is>
+      </c>
       <c r="J11" t="inlineStr">
         <is>
           <t>0.5814±0.0182</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>0.5649±0.0139</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>0.5542±0.0086</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>0.5404±0.0100</t>
+        </is>
+      </c>
       <c r="N11" t="inlineStr">
         <is>
           <t>0.6117±0.0098</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>0.6044±0.0090</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>0.5955±0.0073</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>0.5647±0.0097</t>
+        </is>
+      </c>
       <c r="R11" t="inlineStr">
         <is>
           <t>0.8082±0.0049</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr"/>
-      <c r="T11" t="inlineStr"/>
-      <c r="U11" t="inlineStr"/>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>0.8069±0.0042</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>0.8002±0.0046</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>0.7762±0.0059</t>
+        </is>
+      </c>
       <c r="V11" t="inlineStr">
         <is>
           <t>0.5134±0.0102</t>
         </is>
       </c>
-      <c r="W11" t="inlineStr"/>
-      <c r="X11" t="inlineStr"/>
-      <c r="Y11" t="inlineStr"/>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>0.5018±0.0089</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>0.4880±0.0090</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>0.4474±0.0109</t>
+        </is>
+      </c>
       <c r="Z11" t="inlineStr">
         <is>
           <t>0.3793±0.0125</t>
         </is>
       </c>
-      <c r="AA11" t="inlineStr"/>
-      <c r="AB11" t="inlineStr"/>
-      <c r="AC11" t="inlineStr"/>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>0.3627±0.0110</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>0.3518±0.0128</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>0.3558±0.0097</t>
+        </is>
+      </c>
       <c r="AD11" t="inlineStr">
         <is>
           <t>0.6016±0.0616</t>
         </is>
       </c>
-      <c r="AE11" t="inlineStr"/>
-      <c r="AF11" t="inlineStr"/>
-      <c r="AG11" t="inlineStr"/>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>0.5999±0.0579</t>
+        </is>
+      </c>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>0.5680±0.0423</t>
+        </is>
+      </c>
+      <c r="AG11" t="inlineStr">
+        <is>
+          <t>0.4446±0.0216</t>
+        </is>
+      </c>
       <c r="AH11" t="inlineStr">
         <is>
           <t>0.3460±0.0121</t>
         </is>
       </c>
-      <c r="AI11" t="inlineStr"/>
-      <c r="AJ11" t="inlineStr"/>
-      <c r="AK11" t="inlineStr"/>
+      <c r="AI11" t="inlineStr">
+        <is>
+          <t>0.3278±0.0090</t>
+        </is>
+      </c>
+      <c r="AJ11" t="inlineStr">
+        <is>
+          <t>0.3201±0.0085</t>
+        </is>
+      </c>
+      <c r="AK11" t="inlineStr">
+        <is>
+          <t>0.3283±0.0087</t>
+        </is>
+      </c>
       <c r="AL11" t="inlineStr">
         <is>
           <t>1.0000±0.0000</t>
         </is>
       </c>
-      <c r="AM11" t="inlineStr"/>
-      <c r="AN11" t="inlineStr"/>
-      <c r="AO11" t="inlineStr"/>
+      <c r="AM11" t="inlineStr">
+        <is>
+          <t>1.0000±0.0000</t>
+        </is>
+      </c>
+      <c r="AN11" t="inlineStr">
+        <is>
+          <t>0.9998±0.0006</t>
+        </is>
+      </c>
+      <c r="AO11" t="inlineStr">
+        <is>
+          <t>0.9951±0.0039</t>
+        </is>
+      </c>
       <c r="AP11" t="inlineStr">
         <is>
           <t>0.6451±0.0088</t>
         </is>
       </c>
-      <c r="AQ11" t="inlineStr"/>
-      <c r="AR11" t="inlineStr"/>
-      <c r="AS11" t="inlineStr"/>
+      <c r="AQ11" t="inlineStr">
+        <is>
+          <t>0.6368±0.0075</t>
+        </is>
+      </c>
+      <c r="AR11" t="inlineStr">
+        <is>
+          <t>0.6246±0.0079</t>
+        </is>
+      </c>
+      <c r="AS11" t="inlineStr">
+        <is>
+          <t>0.5924±0.0086</t>
+        </is>
+      </c>
       <c r="AT11" t="inlineStr">
         <is>
           <t>0.7330±0.0055</t>
         </is>
       </c>
-      <c r="AU11" t="inlineStr"/>
-      <c r="AV11" t="inlineStr"/>
-      <c r="AW11" t="inlineStr"/>
+      <c r="AU11" t="inlineStr">
+        <is>
+          <t>0.7393±0.0073</t>
+        </is>
+      </c>
+      <c r="AV11" t="inlineStr">
+        <is>
+          <t>0.7243±0.0138</t>
+        </is>
+      </c>
+      <c r="AW11" t="inlineStr">
+        <is>
+          <t>0.6603±0.0143</t>
+        </is>
+      </c>
       <c r="AX11" t="inlineStr">
         <is>
           <t>0.5764±0.0161</t>
         </is>
       </c>
-      <c r="AY11" t="inlineStr"/>
-      <c r="AZ11" t="inlineStr"/>
-      <c r="BA11" t="inlineStr"/>
+      <c r="AY11" t="inlineStr">
+        <is>
+          <t>0.5594±0.0121</t>
+        </is>
+      </c>
+      <c r="AZ11" t="inlineStr">
+        <is>
+          <t>0.5491±0.0093</t>
+        </is>
+      </c>
+      <c r="BA11" t="inlineStr">
+        <is>
+          <t>0.5374±0.0103</t>
+        </is>
+      </c>
       <c r="BB11" t="inlineStr">
         <is>
           <t>0.2201±0.0155</t>
         </is>
       </c>
-      <c r="BC11" t="inlineStr"/>
-      <c r="BD11" t="inlineStr"/>
-      <c r="BE11" t="inlineStr"/>
+      <c r="BC11" t="inlineStr">
+        <is>
+          <t>0.1849±0.0154</t>
+        </is>
+      </c>
+      <c r="BD11" t="inlineStr">
+        <is>
+          <t>0.1487±0.0164</t>
+        </is>
+      </c>
+      <c r="BE11" t="inlineStr">
+        <is>
+          <t>0.0799±0.0161</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1916,113 +3596,281 @@
           <t>0.8898±0.0128</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>0.8847±0.0124</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>0.8710±0.0182</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>0.8217±0.0168</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr">
         <is>
           <t>0.7570±0.0106</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>0.7539±0.0076</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>0.7489±0.0096</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>0.7234±0.0133</t>
+        </is>
+      </c>
       <c r="J12" t="inlineStr">
         <is>
           <t>0.4481±0.0171</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>0.4611±0.0154</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>0.4556±0.0156</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>0.4287±0.0159</t>
+        </is>
+      </c>
       <c r="N12" t="inlineStr">
         <is>
           <t>0.5368±0.0131</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>0.5456±0.0109</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>0.5383±0.0114</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>0.5066±0.0140</t>
+        </is>
+      </c>
       <c r="R12" t="inlineStr">
         <is>
           <t>0.7930±0.0056</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr"/>
-      <c r="T12" t="inlineStr"/>
-      <c r="U12" t="inlineStr"/>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>0.7952±0.0052</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>0.7933±0.0060</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>0.7835±0.0050</t>
+        </is>
+      </c>
       <c r="V12" t="inlineStr">
         <is>
           <t>0.4227±0.0121</t>
         </is>
       </c>
-      <c r="W12" t="inlineStr"/>
-      <c r="X12" t="inlineStr"/>
-      <c r="Y12" t="inlineStr"/>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>0.4333±0.0112</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>0.4264±0.0123</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>0.3953±0.0134</t>
+        </is>
+      </c>
       <c r="Z12" t="inlineStr">
         <is>
           <t>0.2637±0.0120</t>
         </is>
       </c>
-      <c r="AA12" t="inlineStr"/>
-      <c r="AB12" t="inlineStr"/>
-      <c r="AC12" t="inlineStr"/>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>0.2718±0.0115</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>0.2713±0.0138</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>0.2720±0.0101</t>
+        </is>
+      </c>
       <c r="AD12" t="inlineStr">
         <is>
           <t>0.5934±0.0745</t>
         </is>
       </c>
-      <c r="AE12" t="inlineStr"/>
-      <c r="AF12" t="inlineStr"/>
-      <c r="AG12" t="inlineStr"/>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>0.5903±0.0697</t>
+        </is>
+      </c>
+      <c r="AF12" t="inlineStr">
+        <is>
+          <t>0.5447±0.0523</t>
+        </is>
+      </c>
+      <c r="AG12" t="inlineStr">
+        <is>
+          <t>0.5556±0.0786</t>
+        </is>
+      </c>
       <c r="AH12" t="inlineStr">
         <is>
           <t>0.2306±0.0089</t>
         </is>
       </c>
-      <c r="AI12" t="inlineStr"/>
-      <c r="AJ12" t="inlineStr"/>
-      <c r="AK12" t="inlineStr"/>
+      <c r="AI12" t="inlineStr">
+        <is>
+          <t>0.2395±0.0090</t>
+        </is>
+      </c>
+      <c r="AJ12" t="inlineStr">
+        <is>
+          <t>0.2373±0.0106</t>
+        </is>
+      </c>
+      <c r="AK12" t="inlineStr">
+        <is>
+          <t>0.2292±0.0097</t>
+        </is>
+      </c>
       <c r="AL12" t="inlineStr">
         <is>
           <t>1.0000±0.0000</t>
         </is>
       </c>
-      <c r="AM12" t="inlineStr"/>
-      <c r="AN12" t="inlineStr"/>
-      <c r="AO12" t="inlineStr"/>
+      <c r="AM12" t="inlineStr">
+        <is>
+          <t>1.0000±0.0000</t>
+        </is>
+      </c>
+      <c r="AN12" t="inlineStr">
+        <is>
+          <t>1.0000±0.0000</t>
+        </is>
+      </c>
+      <c r="AO12" t="inlineStr">
+        <is>
+          <t>1.0000±0.0000</t>
+        </is>
+      </c>
       <c r="AP12" t="inlineStr">
         <is>
           <t>0.5689±0.0119</t>
         </is>
       </c>
-      <c r="AQ12" t="inlineStr"/>
-      <c r="AR12" t="inlineStr"/>
-      <c r="AS12" t="inlineStr"/>
+      <c r="AQ12" t="inlineStr">
+        <is>
+          <t>0.5782±0.0110</t>
+        </is>
+      </c>
+      <c r="AR12" t="inlineStr">
+        <is>
+          <t>0.5721±0.0130</t>
+        </is>
+      </c>
+      <c r="AS12" t="inlineStr">
+        <is>
+          <t>0.5444±0.0129</t>
+        </is>
+      </c>
       <c r="AT12" t="inlineStr">
         <is>
           <t>0.7696±0.0084</t>
         </is>
       </c>
-      <c r="AU12" t="inlineStr"/>
-      <c r="AV12" t="inlineStr"/>
-      <c r="AW12" t="inlineStr"/>
+      <c r="AU12" t="inlineStr">
+        <is>
+          <t>0.7673±0.0083</t>
+        </is>
+      </c>
+      <c r="AV12" t="inlineStr">
+        <is>
+          <t>0.7659±0.0107</t>
+        </is>
+      </c>
+      <c r="AW12" t="inlineStr">
+        <is>
+          <t>0.7501±0.0138</t>
+        </is>
+      </c>
       <c r="AX12" t="inlineStr">
         <is>
           <t>0.4514±0.0142</t>
         </is>
       </c>
-      <c r="AY12" t="inlineStr"/>
-      <c r="AZ12" t="inlineStr"/>
-      <c r="BA12" t="inlineStr"/>
+      <c r="AY12" t="inlineStr">
+        <is>
+          <t>0.4640±0.0136</t>
+        </is>
+      </c>
+      <c r="AZ12" t="inlineStr">
+        <is>
+          <t>0.4568±0.0153</t>
+        </is>
+      </c>
+      <c r="BA12" t="inlineStr">
+        <is>
+          <t>0.4276±0.0172</t>
+        </is>
+      </c>
       <c r="BB12" t="inlineStr">
         <is>
           <t>0.0819±0.0095</t>
         </is>
       </c>
-      <c r="BC12" t="inlineStr"/>
-      <c r="BD12" t="inlineStr"/>
-      <c r="BE12" t="inlineStr"/>
+      <c r="BC12" t="inlineStr">
+        <is>
+          <t>0.0952±0.0143</t>
+        </is>
+      </c>
+      <c r="BD12" t="inlineStr">
+        <is>
+          <t>0.0923±0.0107</t>
+        </is>
+      </c>
+      <c r="BE12" t="inlineStr">
+        <is>
+          <t>0.0753±0.0156</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">

</xml_diff>